<commit_message>
Clarify Task B scope and evidence
</commit_message>
<xml_diff>
--- a/outputs/github-org-iac-future-rollout/github-org-iac-future-rollout-vi.xlsx
+++ b/outputs/github-org-iac-future-rollout/github-org-iac-future-rollout-vi.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="R23b00eeef0054644"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IaC nhưng Manual UI" sheetId="2" r:id="R81f66b3fb4594e3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lộ trình" sheetId="3" r:id="R3604fcb2b966446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiểm thử &amp; rủi ro" sheetId="4" r:id="R340a60e3d5d64340"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="Rebdcba8f80f948fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IaC nhưng Manual UI" sheetId="2" r:id="R68d5a35b92ce4b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lộ trình" sheetId="3" r:id="R31cd41a56bf841fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiểm thử &amp; rủi ro" sheetId="4" r:id="R81ff6aea47154f70"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="13">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -46,12 +46,6 @@
       <x:b/>
       <x:sz val="10"/>
       <x:color rgb="FF17365D"/>
-      <x:name val="Arial"/>
-    </x:font>
-    <x:font>
-      <x:b/>
-      <x:sz val="10"/>
-      <x:color rgb="FF7F6000"/>
       <x:name val="Arial"/>
     </x:font>
     <x:font>
@@ -95,7 +89,7 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -109,17 +103,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFF2CC"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFCE4D6"/>
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -225,77 +214,88 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top"/>
+      <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="200" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="12">
+  <x:dxfs count="15">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF385723"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -353,6 +353,17 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF385723"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
@@ -379,6 +390,17 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF385723"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -446,7 +468,7 @@
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>Bằng chứng PoC hiện tại</a:t>
+              <a:t>Bằng chứng Task 2 hiện tại</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -588,7 +610,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R271ec8037a0d45db"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R297589f19ea841c5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -614,14 +636,14 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RolloutRoadmap" displayName="RolloutRoadmap" ref="A4:I9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
-    <x:tableColumn id="1" name="Phase"/>
+    <x:tableColumn id="1" name="Bước"/>
     <x:tableColumn id="2" name="Mục tiêu"/>
     <x:tableColumn id="3" name="Phạm vi"/>
-    <x:tableColumn id="4" name="Deliverable"/>
-    <x:tableColumn id="5" name="Exit criteria"/>
+    <x:tableColumn id="4" name="Bằng chứng cần lưu"/>
+    <x:tableColumn id="5" name="Điều kiện hoàn tất"/>
     <x:tableColumn id="6" name="Owner"/>
-    <x:tableColumn id="7" name="Tuần"/>
-    <x:tableColumn id="8" name="Bắt đầu"/>
+    <x:tableColumn id="7" name="Ước lượng"/>
+    <x:tableColumn id="8" name="Thứ tự"/>
     <x:tableColumn id="9" name="Trạng thái"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -632,8 +654,8 @@
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DecisionTests" displayName="DecisionTests" ref="A8:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="ID"/>
-    <x:tableColumn id="2" name="Case"/>
-    <x:tableColumn id="3" name="Rủi ro được kiểm"/>
+    <x:tableColumn id="2" name="Yêu cầu"/>
+    <x:tableColumn id="3" name="Phạm vi"/>
     <x:tableColumn id="4" name="Bằng chứng hiện tại"/>
     <x:tableColumn id="5" name="Trạng thái"/>
     <x:tableColumn id="6" name="Owner"/>
@@ -646,13 +668,13 @@
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RiskControls" displayName="RiskControls" ref="A24:G30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
-    <x:tableColumn id="1" name="Rủi ro"/>
-    <x:tableColumn id="2" name="Khả năng"/>
-    <x:tableColumn id="3" name="Tác động"/>
-    <x:tableColumn id="4" name="Kiểm soát"/>
-    <x:tableColumn id="5" name="Khi nào"/>
+    <x:tableColumn id="1" name="Limitation"/>
+    <x:tableColumn id="2" name="Liên quan"/>
+    <x:tableColumn id="3" name="Quan sát"/>
+    <x:tableColumn id="4" name="Cách ghi report"/>
+    <x:tableColumn id="5" name="Ảnh hưởng"/>
     <x:tableColumn id="6" name="Owner"/>
-    <x:tableColumn id="7" name="Mức còn lại"/>
+    <x:tableColumn id="7" name="Trạng thái"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -874,7 +896,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
-        <x:v>GitHub Organization IaC – định hướng triển khai</x:v>
+        <x:v>Task 2 – GitHub Org Teams bằng Terraform</x:v>
       </x:c>
       <x:c r="B1" s="41"/>
       <x:c r="C1" s="41"/>
@@ -892,7 +914,7 @@
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Tóm tắt cho team lead | Sandbox xbrain-org-poc | Cập nhật 2026-09-30</x:v>
+        <x:v>Phạm vi: team và direct team membership | Không bao gồm Org Members | Cập nhật 2026-10-01</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -925,72 +947,72 @@
         <x:v>Số case</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5" ht="24" hidden="0" customHeight="1">
       <x:c r="A5" s="12" t="str">
-        <x:v>Khuyến nghị</x:v>
+        <x:v>Phạm vi gốc</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
-        <x:v>Go có điều kiện</x:v>
+        <x:v>Create/update/delete team; add/remove member; đổi team role</x:v>
       </x:c>
       <x:c r="H5" s="27" t="str">
         <x:v>Đạt</x:v>
       </x:c>
       <x:c r="I5" s="31" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Đạt")</x:f>
-        <x:v>3</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A6" s="12" t="str">
-        <x:v>Đã chứng minh</x:v>
+        <x:v>Đã chứng minh live</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Tạo team + membership; plan sau apply không đổi</x:v>
+        <x:v>Create team + owner direct membership; plan sau apply không đổi</x:v>
       </x:c>
       <x:c r="H6" s="28" t="str">
         <x:v>Đạt một phần</x:v>
       </x:c>
       <x:c r="I6" s="32" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Đạt một phần")</x:f>
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>Đang quản lý</x:v>
+        <x:v>Chưa chứng minh live</x:v>
       </x:c>
       <x:c r="B7" s="13" t="str">
-        <x:v>poc-devops / owner maintainer</x:v>
+        <x:v>Update/delete team; add/remove/đổi role member thường</x:v>
       </x:c>
       <x:c r="H7" s="28" t="str">
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="I7" s="32" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Chưa chạy")</x:f>
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A8" s="12" t="str">
-        <x:v>Chưa chứng minh</x:v>
+        <x:v>Ngoài phạm vi</x:v>
       </x:c>
       <x:c r="B8" s="13" t="str">
-        <x:v>Update role user thường, drift, import, cleanup</x:v>
+        <x:v>Invite, đổi org role, remove org member – Task 1 của Hoàng</x:v>
       </x:c>
       <x:c r="H8" s="28" t="str">
         <x:v>Chặn</x:v>
       </x:c>
       <x:c r="I8" s="32" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Chặn")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
-        <x:v>Production</x:v>
+        <x:v>Kết luận</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>Chưa sẵn sàng</x:v>
+        <x:v>Khả thi bước đầu; chưa đủ dữ liệu cho toàn bộ lifecycle</x:v>
       </x:c>
     </x:row>
     <x:row r="10"/>
@@ -1026,7 +1048,7 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="27" t="str">
-        <x:v>Create &amp; convergence</x:v>
+        <x:v>Create + convergence</x:v>
       </x:c>
       <x:c r="B13" s="27" t="str">
         <x:v>Đạt</x:v>
@@ -1035,93 +1057,93 @@
         <x:v>2 add; follow-up plan = 0</x:v>
       </x:c>
       <x:c r="D13" s="27" t="str">
-        <x:v>Giữ no-change plan</x:v>
+        <x:v>Giữ bằng chứng</x:v>
       </x:c>
       <x:c r="E13" s="27" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="F13" s="27" t="str">
-        <x:v>Tiếp tục</x:v>
+        <x:v>Đã chứng minh</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="28" t="str">
-        <x:v>Membership boundary</x:v>
+        <x:v>Update team</x:v>
       </x:c>
       <x:c r="B14" s="28" t="str">
+        <x:v>Chưa chạy</x:v>
+      </x:c>
+      <x:c r="C14" s="28" t="str">
+        <x:v>Mới có preview</x:v>
+      </x:c>
+      <x:c r="D14" s="28" t="str">
+        <x:v>Apply + UI/state + no-change plan</x:v>
+      </x:c>
+      <x:c r="E14" s="28" t="str">
+        <x:v>Task 2</x:v>
+      </x:c>
+      <x:c r="F14" s="28" t="str">
+        <x:v>Cần chạy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" hidden="0" customHeight="1">
+      <x:c r="A15" s="28" t="str">
+        <x:v>Team membership</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="str">
         <x:v>Đạt một phần</x:v>
       </x:c>
-      <x:c r="C14" s="28" t="str">
-        <x:v>Outsider 404; pending chưa thử</x:v>
-      </x:c>
-      <x:c r="D14" s="28" t="str">
-        <x:v>Pending + active user</x:v>
-      </x:c>
-      <x:c r="E14" s="28" t="str">
-        <x:v>Org owner</x:v>
-      </x:c>
-      <x:c r="F14" s="28" t="str">
-        <x:v>Tiếp tục có kiểm soát</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="15" hidden="0" customHeight="1">
-      <x:c r="A15" s="28" t="str">
-        <x:v>Full lifecycle</x:v>
-      </x:c>
-      <x:c r="B15" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
-      </x:c>
       <x:c r="C15" s="28" t="str">
-        <x:v>Chưa có update/remove/import</x:v>
+        <x:v>Owner maintainer đạt; user thường chưa thử</x:v>
       </x:c>
       <x:c r="D15" s="28" t="str">
-        <x:v>Hoàn tất edge cases</x:v>
+        <x:v>Add/role/remove với active member</x:v>
       </x:c>
       <x:c r="E15" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="F15" s="28" t="str">
-        <x:v>Chưa production</x:v>
+        <x:v>Cần chạy</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="28" t="str">
-        <x:v>State &amp; review</x:v>
+        <x:v>Delete team</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>State local</x:v>
+        <x:v>Chưa có live plan/apply</x:v>
       </x:c>
       <x:c r="D16" s="28" t="str">
-        <x:v>Remote state + locking + PR</x:v>
+        <x:v>Xóa team disposable an toàn</x:v>
       </x:c>
       <x:c r="E16" s="28" t="str">
-        <x:v>Platform lead</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="F16" s="28" t="str">
-        <x:v>Chưa production</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="15" hidden="0" customHeight="1">
+        <x:v>Cần chạy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="28" t="str">
-        <x:v>Credential model</x:v>
+        <x:v>Org member lifecycle</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>Chặn</x:v>
+        <x:v>Ngoài phạm vi</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>GCM token thiếu admin:org</x:v>
+        <x:v>Không có resource mutation trong code</x:v>
       </x:c>
       <x:c r="D17" s="28" t="str">
-        <x:v>GitHub App/PAT đúng quyền</x:v>
+        <x:v>Task 1 cung cấp active member</x:v>
       </x:c>
       <x:c r="E17" s="28" t="str">
-        <x:v>Org owner</x:v>
+        <x:v>Hoàng</x:v>
       </x:c>
       <x:c r="F17" s="28" t="str">
-        <x:v>Phải xử lý</x:v>
+        <x:v>Phụ thuộc</x:v>
       </x:c>
     </x:row>
     <x:row r="18"/>
@@ -1141,13 +1163,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>Hoàn tất lifecycle trên sandbox</x:v>
+        <x:v>Update team trên sandbox</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>Role, drift, import, remove, cleanup</x:v>
+        <x:v>Name/description/setting; giữ resource identity</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>Bắt buộc trước pilot</x:v>
+        <x:v>Ghi plan, UI/state và no-change plan</x:v>
       </x:c>
       <x:c r="E21" t="str"/>
       <x:c r="F21" t="str"/>
@@ -1157,13 +1179,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B22" s="11" t="str">
-        <x:v>Tách bootstrap khỏi steady state</x:v>
+        <x:v>Nhận active member từ Task 1</x:v>
       </x:c>
       <x:c r="C22" s="11" t="str">
-        <x:v>UI/API mời org member; Terraform quản lý team</x:v>
+        <x:v>Task 2 không invite hoặc đổi org role</x:v>
       </x:c>
       <x:c r="D22" s="11" t="str">
-        <x:v>Giữ boundary rõ</x:v>
+        <x:v>Giữ ranh giới ownership</x:v>
       </x:c>
       <x:c r="E22" t="str"/>
       <x:c r="F22" t="str"/>
@@ -1173,13 +1195,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="11" t="str">
-        <x:v>Chuẩn hóa credential</x:v>
+        <x:v>Test team membership</x:v>
       </x:c>
       <x:c r="C23" s="11" t="str">
-        <x:v>GitHub App hoặc PAT ngắn hạn đúng quyền</x:v>
+        <x:v>Add, member ↔ maintainer, remove</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
-        <x:v>Không dùng token cá nhân dài hạn</x:v>
+        <x:v>Org membership phải còn nguyên</x:v>
       </x:c>
       <x:c r="E23" t="str"/>
       <x:c r="F23" t="str"/>
@@ -1189,13 +1211,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B24" s="11" t="str">
-        <x:v>Chuyển state ra backend có locking</x:v>
+        <x:v>Test delete team disposable</x:v>
       </x:c>
       <x:c r="C24" s="11" t="str">
-        <x:v>Bảo vệ state và chống apply đồng thời</x:v>
+        <x:v>Xem destructive plan trước apply</x:v>
       </x:c>
       <x:c r="D24" s="11" t="str">
-        <x:v>Bắt buộc trước nhiều admin</x:v>
+        <x:v>Xác nhận state và GitHub</x:v>
       </x:c>
       <x:c r="E24" t="str"/>
       <x:c r="F24" t="str"/>
@@ -1205,13 +1227,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B25" s="11" t="str">
-        <x:v>Đưa thay đổi qua PR</x:v>
+        <x:v>Chốt limitation</x:v>
       </x:c>
       <x:c r="C25" s="11" t="str">
-        <x:v>Plan, review, apply có kiểm soát</x:v>
+        <x:v>Ghi behavior thực tế; tách phần mở rộng</x:v>
       </x:c>
       <x:c r="D25" s="11" t="str">
-        <x:v>Audit và rollback rõ</x:v>
+        <x:v>Đủ bằng chứng cho Task 2</x:v>
       </x:c>
       <x:c r="E25" t="str"/>
       <x:c r="F25" t="str"/>
@@ -1304,17 +1326,20 @@
       <x:formula>"Đạt"</x:formula>
     </x:cfRule>
     <x:cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <x:formula>"Hoàn tất"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <x:formula>"Đạt một phần"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <x:cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <x:formula>"Chưa chạy"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
+    <x:cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <x:formula>"Chặn"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f3b79914a4444d6"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9974298fc3a64c1d"/>
 </x:worksheet>
 </file>
 
@@ -1335,7 +1360,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
-        <x:v>IaC nhưng vẫn cần Manual UI</x:v>
+        <x:v>Task 2: IaC nhưng vẫn cần Manual UI</x:v>
       </x:c>
       <x:c r="B1" s="41"/>
       <x:c r="C1" s="41"/>
@@ -1345,7 +1370,7 @@
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>So sánh trade-off để chọn đúng công cụ cho từng loại thay đổi</x:v>
+        <x:v>So sánh trong phạm vi team và direct team membership</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1391,7 +1416,7 @@
         <x:v>Dễ lệch chuẩn khi số lượng tăng</x:v>
       </x:c>
       <x:c r="F5" s="35" t="str">
-        <x:v>IaC chính</x:v>
+        <x:v>Đánh giá sau PoC</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="62" hidden="0" customHeight="1">
@@ -1411,7 +1436,7 @@
         <x:v>Khó thấy ý định trước thay đổi</x:v>
       </x:c>
       <x:c r="F6" s="36" t="str">
-        <x:v>IaC chính</x:v>
+        <x:v>IaC phù hợp nếu lifecycle đạt</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" hidden="0" customHeight="1">
@@ -1431,7 +1456,7 @@
         <x:v>Không tự chỉ ra chênh lệch với chuẩn</x:v>
       </x:c>
       <x:c r="F7" s="36" t="str">
-        <x:v>IaC chính</x:v>
+        <x:v>Kiểm thử mở rộng</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="62" hidden="0" customHeight="1">
@@ -1451,7 +1476,7 @@
         <x:v>Khó lặp lại và dễ thiếu bằng chứng</x:v>
       </x:c>
       <x:c r="F8" s="36" t="str">
-        <x:v>UI bổ trợ</x:v>
+        <x:v>Ngoài Task 2</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="62" hidden="0" customHeight="1">
@@ -1491,7 +1516,7 @@
         <x:v>Click nhầm có thể ảnh hưởng rộng</x:v>
       </x:c>
       <x:c r="F10" s="36" t="str">
-        <x:v>IaC + checklist</x:v>
+        <x:v>Kiểm thử mở rộng</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" hidden="0" customHeight="1">
@@ -1511,7 +1536,7 @@
         <x:v>Khó kiểm soát ở quy mô lớn</x:v>
       </x:c>
       <x:c r="F11" s="36" t="str">
-        <x:v>IaC chính</x:v>
+        <x:v>Đánh giá sau live test</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" hidden="0" customHeight="1">
@@ -1531,14 +1556,14 @@
         <x:v>Tiếp tục duy trì thủ công</x:v>
       </x:c>
       <x:c r="F12" s="36" t="str">
-        <x:v>IaC theo từng đợt</x:v>
+        <x:v>Ngoài yêu cầu gốc</x:v>
       </x:c>
     </x:row>
     <x:row r="13"/>
     <x:row r="14"/>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="6" t="str">
-        <x:v>Nguyên tắc vận hành đề xuất</x:v>
+        <x:v>Ranh giới áp dụng trong PoC</x:v>
       </x:c>
       <x:c r="B15" s="7"/>
       <x:c r="C15" s="7"/>
@@ -1548,10 +1573,10 @@
     </x:row>
     <x:row r="16" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A16" s="10" t="str">
-        <x:v>Steady state</x:v>
+        <x:v>Trong PoC</x:v>
       </x:c>
       <x:c r="B16" s="11" t="str">
-        <x:v>Terraform là nguồn chuẩn cho team và direct membership.</x:v>
+        <x:v>Terraform quản lý team và direct team membership đã khai báo.</x:v>
       </x:c>
       <x:c r="C16" t="str"/>
       <x:c r="D16" t="str"/>
@@ -1560,10 +1585,10 @@
     </x:row>
     <x:row r="17" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A17" s="10" t="str">
-        <x:v>Bootstrap</x:v>
+        <x:v>Phụ thuộc Task 1</x:v>
       </x:c>
       <x:c r="B17" s="11" t="str">
-        <x:v>UI/API chỉ dùng để tạo credential, mời org member và xử lý điều kiện ban đầu.</x:v>
+        <x:v>Org member phải tồn tại và active trước khi Task 2 thêm vào team.</x:v>
       </x:c>
       <x:c r="C17" t="str"/>
       <x:c r="D17" t="str"/>
@@ -1572,22 +1597,22 @@
     </x:row>
     <x:row r="18" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A18" s="10" t="str">
-        <x:v>Break-glass</x:v>
+        <x:v>Manual UI</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
-        <x:v>Cho phép UI khi khẩn cấp, nhưng phải tạo PR reconcile trong ngày làm việc kế tiếp.</x:v>
+        <x:v>Dùng để đối chiếu kết quả và xử lý bước thuộc Task 1; không tính là bằng chứng IaC Task 2.</x:v>
       </x:c>
       <x:c r="C18" t="str"/>
       <x:c r="D18" t="str"/>
       <x:c r="E18" t="str"/>
       <x:c r="F18" t="str"/>
     </x:row>
-    <x:row r="19" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="19" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A19" s="10" t="str">
         <x:v>Ngoài phạm vi</x:v>
       </x:c>
       <x:c r="B19" s="11" t="str">
-        <x:v>IdP/SCIM và repository permission có owner/quy trình riêng.</x:v>
+        <x:v>Org membership lifecycle, repository permission, IdP/SCIM và production rollout.</x:v>
       </x:c>
       <x:c r="C19" t="str"/>
       <x:c r="D19" t="str"/>
@@ -1597,7 +1622,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf444b9e9ab0b49a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref8d42a97c444141"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1622,7 +1647,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
-        <x:v>Lộ trình từ PoC đến vận hành</x:v>
+        <x:v>Các bước hoàn tất Task 2</x:v>
       </x:c>
       <x:c r="B1" s="41"/>
       <x:c r="C1" s="41"/>
@@ -1635,7 +1660,7 @@
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Mỗi phase chỉ chuyển tiếp khi exit criteria đã có bằng chứng</x:v>
+        <x:v>Chỉ tính hoàn tất khi có plan/apply, state và kiểm tra thực tế trên GitHub</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1649,7 +1674,7 @@
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="23" t="str">
-        <x:v>Phase</x:v>
+        <x:v>Bước</x:v>
       </x:c>
       <x:c r="B4" s="23" t="str">
         <x:v>Mục tiêu</x:v>
@@ -1658,19 +1683,19 @@
         <x:v>Phạm vi</x:v>
       </x:c>
       <x:c r="D4" s="23" t="str">
-        <x:v>Deliverable</x:v>
+        <x:v>Bằng chứng cần lưu</x:v>
       </x:c>
       <x:c r="E4" s="23" t="str">
-        <x:v>Exit criteria</x:v>
+        <x:v>Điều kiện hoàn tất</x:v>
       </x:c>
       <x:c r="F4" s="23" t="str">
         <x:v>Owner</x:v>
       </x:c>
       <x:c r="G4" s="23" t="str">
-        <x:v>Tuần</x:v>
+        <x:v>Ước lượng</x:v>
       </x:c>
       <x:c r="H4" s="23" t="str">
-        <x:v>Bắt đầu</x:v>
+        <x:v>Thứ tự</x:v>
       </x:c>
       <x:c r="I4" s="23" t="str">
         <x:v>Trạng thái</x:v>
@@ -1678,58 +1703,58 @@
     </x:row>
     <x:row r="5" ht="56" hidden="0" customHeight="1">
       <x:c r="A5" s="27" t="str">
-        <x:v>0. PoC</x:v>
+        <x:v>0. Baseline</x:v>
       </x:c>
       <x:c r="B5" s="27" t="str">
-        <x:v>Chứng minh lifecycle</x:v>
+        <x:v>Create + convergence</x:v>
       </x:c>
       <x:c r="C5" s="27" t="str">
-        <x:v>Team + direct membership</x:v>
+        <x:v>1 team + owner membership</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Evidence create/update/drift/import/remove</x:v>
+        <x:v>Plan/apply/API/no-change plan</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Không có diff lặp; cleanup an toàn</x:v>
+        <x:v>Đã khớp state và GitHub</x:v>
       </x:c>
       <x:c r="F5" s="27" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G5" s="31" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H5" s="31" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="I5" s="27" t="str">
-        <x:v>Đang làm</x:v>
+        <x:v>Hoàn tất</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="56" hidden="0" customHeight="1">
       <x:c r="A6" s="28" t="str">
-        <x:v>1. Hardening</x:v>
+        <x:v>1. Update team</x:v>
       </x:c>
       <x:c r="B6" s="28" t="str">
-        <x:v>Chuẩn hóa vận hành</x:v>
+        <x:v>Kiểm tra update</x:v>
       </x:c>
       <x:c r="C6" s="28" t="str">
-        <x:v>Credential, state, review</x:v>
+        <x:v>Name/description/setting</x:v>
       </x:c>
       <x:c r="D6" s="28" t="str">
-        <x:v>GitHub App/PAT model; remote state; runbook</x:v>
+        <x:v>Plan/apply/UI/state/no-change</x:v>
       </x:c>
       <x:c r="E6" s="28" t="str">
-        <x:v>Locking và least privilege đạt</x:v>
+        <x:v>Không destroy ngoài dự kiến</x:v>
       </x:c>
       <x:c r="F6" s="28" t="str">
-        <x:v>Platform lead</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G6" s="32" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H6" s="32" t="n">
         <x:f>H5+G5</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="I6" s="28" t="str">
         <x:v>Chưa bắt đầu</x:v>
@@ -1737,59 +1762,59 @@
     </x:row>
     <x:row r="7" ht="56" hidden="0" customHeight="1">
       <x:c r="A7" s="28" t="str">
-        <x:v>2. Pilot</x:v>
+        <x:v>2. Team membership</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
-        <x:v>Chạy với scope nhỏ</x:v>
+        <x:v>Kiểm tra add/role/remove</x:v>
       </x:c>
       <x:c r="C7" s="28" t="str">
-        <x:v>2–3 team không critical</x:v>
+        <x:v>Active ordinary member</x:v>
       </x:c>
       <x:c r="D7" s="28" t="str">
-        <x:v>PR workflow và audit evidence</x:v>
+        <x:v>Plan/apply/API/state từng bước</x:v>
       </x:c>
       <x:c r="E7" s="28" t="str">
-        <x:v>2 chu kỳ thay đổi ổn định</x:v>
+        <x:v>Org member không bị thay đổi</x:v>
       </x:c>
       <x:c r="F7" s="28" t="str">
-        <x:v>Platform + team lead</x:v>
+        <x:v>Task 2 + Task 1</x:v>
       </x:c>
       <x:c r="G7" s="32" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H7" s="32" t="n">
         <x:f>H6+G6</x:f>
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="I7" s="28" t="str">
-        <x:v>Chưa bắt đầu</x:v>
+        <x:v>Chặn</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="56" hidden="0" customHeight="1">
       <x:c r="A8" s="28" t="str">
-        <x:v>3. Migration</x:v>
+        <x:v>3. Delete team</x:v>
       </x:c>
       <x:c r="B8" s="28" t="str">
-        <x:v>Đưa team hiện hữu vào IaC</x:v>
+        <x:v>Kiểm tra delete</x:v>
       </x:c>
       <x:c r="C8" s="28" t="str">
-        <x:v>Import theo từng đợt</x:v>
+        <x:v>Team disposable</x:v>
       </x:c>
       <x:c r="D8" s="28" t="str">
-        <x:v>Catalog team/membership có owner</x:v>
+        <x:v>Destructive plan đã review</x:v>
       </x:c>
       <x:c r="E8" s="28" t="str">
-        <x:v>Import không gây update ngoài dự kiến</x:v>
+        <x:v>Remote và state sạch</x:v>
       </x:c>
       <x:c r="F8" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G8" s="32" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H8" s="32" t="n">
         <x:f>H7+G7</x:f>
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="I8" s="28" t="str">
         <x:v>Chưa bắt đầu</x:v>
@@ -1797,27 +1822,29 @@
     </x:row>
     <x:row r="9" ht="56" hidden="0" customHeight="1">
       <x:c r="A9" s="28" t="str">
-        <x:v>4. BAU</x:v>
+        <x:v>4. Kết luận</x:v>
       </x:c>
       <x:c r="B9" s="28" t="str">
-        <x:v>Vận hành thường xuyên</x:v>
+        <x:v>Chốt limitation</x:v>
       </x:c>
       <x:c r="C9" s="28" t="str">
-        <x:v>Team lifecycle chuẩn</x:v>
+        <x:v>Đúng yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D9" s="28" t="str">
-        <x:v>SLA, review định kỳ, break-glass</x:v>
+        <x:v>Bảng kết quả + behavior</x:v>
       </x:c>
       <x:c r="E9" s="28" t="str">
-        <x:v>Không còn thay đổi UI không reconcile</x:v>
+        <x:v>Không dùng case dự kiến làm evidence</x:v>
       </x:c>
       <x:c r="F9" s="28" t="str">
-        <x:v>Platform ops</x:v>
-      </x:c>
-      <x:c r="G9" s="32"/>
+        <x:v>Task 2</x:v>
+      </x:c>
+      <x:c r="G9" s="32" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="H9" s="32" t="n">
         <x:f>H8+G8</x:f>
-        <x:v>12</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I9" s="28" t="str">
         <x:v>Chưa bắt đầu</x:v>
@@ -1851,60 +1878,63 @@
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="27" t="str">
-        <x:v>Remote state + locking</x:v>
+        <x:v>Active ordinary member</x:v>
       </x:c>
       <x:c r="B14" s="27" t="str">
-        <x:v>Tránh mất state và apply đồng thời</x:v>
+        <x:v>Cần test add/role/remove team membership</x:v>
       </x:c>
       <x:c r="C14" s="27" t="str">
-        <x:v>Bắt buộc trước Pilot</x:v>
+        <x:v>Nhận từ Task 1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="28" t="str">
-        <x:v>Credential tách cá nhân</x:v>
+        <x:v>Plan trước destructive apply</x:v>
       </x:c>
       <x:c r="B15" s="28" t="str">
-        <x:v>Giảm phụ thuộc owner/PAT cá nhân</x:v>
+        <x:v>Delete/remove là yêu cầu gốc nhưng có tác động thật</x:v>
       </x:c>
       <x:c r="C15" s="28" t="str">
-        <x:v>Bắt buộc trước BAU</x:v>
+        <x:v>Bắt buộc</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="28" t="str">
-        <x:v>PR + plan review</x:v>
+        <x:v>UI/API + state + no-change plan</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
-        <x:v>Kiểm soát destroy/replace và audit</x:v>
+        <x:v>Một apply thành công chưa đủ chứng minh hội tụ</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>Bắt buộc trước Pilot</x:v>
+        <x:v>Bắt buộc mỗi flow</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="28" t="str">
-        <x:v>Runbook nested deletion</x:v>
+        <x:v>Tách planned và verified</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>Parent delete có thể cascade ngoài state</x:v>
+        <x:v>Tránh trình bày kỳ vọng như kết quả thực tế</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>Bắt buộc trước Migration</x:v>
+        <x:v>Bắt buộc trong report</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="I5:I9">
-    <x:cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
       <x:formula>"Đạt"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="5" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+      <x:formula>"Hoàn tất"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="7" priority="3" operator="equal">
       <x:formula>"Đạt một phần"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+    <x:cfRule type="cellIs" dxfId="8" priority="4" operator="equal">
       <x:formula>"Chưa chạy"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="7" priority="4" operator="equal">
+    <x:cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
       <x:formula>"Chặn"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -1915,7 +1945,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06315137d88e4f77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e4796a130dd4252"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1938,7 +1968,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
-        <x:v>Kiểm thử và rủi ro quyết định</x:v>
+        <x:v>Bằng chứng và phần việc còn lại</x:v>
       </x:c>
       <x:c r="B1" s="41"/>
       <x:c r="C1" s="41"/>
@@ -1949,7 +1979,7 @@
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Chỉ giữ các case ảnh hưởng trực tiếp đến quyết định Go/No-go</x:v>
+        <x:v>Live = đã plan/apply và đối chiếu GitHub/state; mock hoặc preview không thay thế live evidence</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1976,19 +2006,19 @@
     <x:row r="5" ht="16.799999237060547" hidden="0" customHeight="1">
       <x:c r="A5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Đạt")</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Đạt một phần")</x:f>
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Chưa chạy")</x:f>
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Chặn")</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="6"/>
@@ -1998,10 +2028,10 @@
         <x:v>ID</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
-        <x:v>Case</x:v>
+        <x:v>Yêu cầu</x:v>
       </x:c>
       <x:c r="C8" s="23" t="str">
-        <x:v>Rủi ro được kiểm</x:v>
+        <x:v>Phạm vi</x:v>
       </x:c>
       <x:c r="D8" s="23" t="str">
         <x:v>Bằng chứng hiện tại</x:v>
@@ -2018,243 +2048,243 @@
     </x:row>
     <x:row r="9" ht="50" hidden="0" customHeight="1">
       <x:c r="A9" s="27" t="str">
-        <x:v>CREATE-01</x:v>
+        <x:v>TEAM-CREATE</x:v>
       </x:c>
       <x:c r="B9" s="27" t="str">
-        <x:v>Create + convergence</x:v>
+        <x:v>Create team</x:v>
       </x:c>
       <x:c r="C9" s="27" t="str">
-        <x:v>Provider/state không ổn định</x:v>
+        <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D9" s="27" t="str">
-        <x:v>2 add; follow-up plan = 0</x:v>
+        <x:v>Live: 2 add; team ID 19806617</x:v>
       </x:c>
       <x:c r="E9" s="27" t="str">
         <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F9" s="27" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G9" s="27" t="str">
-        <x:v>Giữ regression check</x:v>
+        <x:v>Giữ evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="50" hidden="0" customHeight="1">
       <x:c r="A10" s="28" t="str">
-        <x:v>AUTH-01</x:v>
+        <x:v>CONVERGE</x:v>
       </x:c>
       <x:c r="B10" s="28" t="str">
-        <x:v>Apply thiếu token</x:v>
+        <x:v>Plan sau apply</x:v>
       </x:c>
       <x:c r="C10" s="28" t="str">
-        <x:v>Anonymous fallback</x:v>
+        <x:v>Xác minh state</x:v>
       </x:c>
       <x:c r="D10" s="28" t="str">
-        <x:v>401 trước mutation</x:v>
+        <x:v>Live: exit 0, no changes</x:v>
       </x:c>
       <x:c r="E10" s="28" t="str">
         <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F10" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G10" s="28" t="str">
-        <x:v>Chuẩn hóa auth wrapper</x:v>
+        <x:v>Lặp lại sau mỗi flow</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="50" hidden="0" customHeight="1">
       <x:c r="A11" s="28" t="str">
-        <x:v>MEMBER-01</x:v>
+        <x:v>TEAM-UPDATE</x:v>
       </x:c>
       <x:c r="B11" s="28" t="str">
-        <x:v>User ngoài org</x:v>
+        <x:v>Update team</x:v>
       </x:c>
       <x:c r="C11" s="28" t="str">
-        <x:v>IaC vô tình mời user</x:v>
+        <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D11" s="28" t="str">
-        <x:v>404; plan exit 1; không mutation</x:v>
+        <x:v>Chỉ có preview; chưa apply</x:v>
       </x:c>
       <x:c r="E11" s="28" t="str">
-        <x:v>Đạt</x:v>
+        <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F11" s="28" t="str">
-        <x:v>Org owner</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G11" s="28" t="str">
-        <x:v>Giữ guard</x:v>
+        <x:v>Apply và verify</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="50" hidden="0" customHeight="1">
       <x:c r="A12" s="28" t="str">
-        <x:v>MEMBER-02</x:v>
+        <x:v>TEAM-DELETE</x:v>
       </x:c>
       <x:c r="B12" s="28" t="str">
-        <x:v>Invitation pending</x:v>
+        <x:v>Delete team</x:v>
       </x:c>
       <x:c r="C12" s="28" t="str">
-        <x:v>Membership tạo trước khi accept</x:v>
+        <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
-        <x:v>Chưa có invitation</x:v>
+        <x:v>Chưa có live plan/apply</x:v>
       </x:c>
       <x:c r="E12" s="28" t="str">
-        <x:v>Chặn</x:v>
+        <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F12" s="28" t="str">
-        <x:v>Org owner</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G12" s="28" t="str">
-        <x:v>Invite phuc776 nhưng chưa accept</x:v>
+        <x:v>Dùng team disposable</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="50" hidden="0" customHeight="1">
       <x:c r="A13" s="28" t="str">
-        <x:v>MEMBER-03</x:v>
+        <x:v>MEMBER-ADD</x:v>
       </x:c>
       <x:c r="B13" s="28" t="str">
-        <x:v>User active</x:v>
+        <x:v>Add member vào team</x:v>
       </x:c>
       <x:c r="C13" s="28" t="str">
-        <x:v>Dependency không hội tụ</x:v>
+        <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D13" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Owner đã được add; user thường chưa thử</x:v>
       </x:c>
       <x:c r="E13" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đạt một phần</x:v>
       </x:c>
       <x:c r="F13" s="28" t="str">
-        <x:v>phuc776</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G13" s="28" t="str">
-        <x:v>Accept rồi plan/apply</x:v>
+        <x:v>Cần active ordinary member</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="50" hidden="0" customHeight="1">
       <x:c r="A14" s="28" t="str">
-        <x:v>ROLE-02</x:v>
+        <x:v>MEMBER-ROLE</x:v>
       </x:c>
       <x:c r="B14" s="28" t="str">
-        <x:v>member ↔ maintainer</x:v>
+        <x:v>Đổi team role</x:v>
       </x:c>
       <x:c r="C14" s="28" t="str">
-        <x:v>Role drift/recreate</x:v>
+        <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D14" s="28" t="str">
-        <x:v>Mock đạt</x:v>
+        <x:v>Mock đạt; chưa có active user thường</x:v>
       </x:c>
       <x:c r="E14" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Chặn</x:v>
       </x:c>
       <x:c r="F14" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G14" s="28" t="str">
-        <x:v>Dùng phuc776</x:v>
+        <x:v>Phụ thuộc Task 1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="50" hidden="0" customHeight="1">
       <x:c r="A15" s="28" t="str">
-        <x:v>TEAM-01</x:v>
+        <x:v>MEMBER-REMOVE</x:v>
       </x:c>
       <x:c r="B15" s="28" t="str">
-        <x:v>Rename/update</x:v>
+        <x:v>Remove member khỏi team</x:v>
       </x:c>
       <x:c r="C15" s="28" t="str">
-        <x:v>Destroy/recreate ngoài ý muốn</x:v>
+        <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D15" s="28" t="str">
-        <x:v>Preview giữ ID 19806617</x:v>
+        <x:v>Chưa có active user thường</x:v>
       </x:c>
       <x:c r="E15" s="28" t="str">
-        <x:v>Đạt một phần</x:v>
+        <x:v>Chặn</x:v>
       </x:c>
       <x:c r="F15" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G15" s="28" t="str">
-        <x:v>Apply sau member active</x:v>
+        <x:v>Phụ thuộc Task 1</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="50" hidden="0" customHeight="1">
       <x:c r="A16" s="28" t="str">
-        <x:v>NEST-01</x:v>
+        <x:v>OUTSIDER</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
-        <x:v>Infra parent + Argo CD child</x:v>
+        <x:v>User chưa thuộc org</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>Sai dependency/privacy</x:v>
+        <x:v>Boundary Task 1/2</x:v>
       </x:c>
       <x:c r="D16" s="28" t="str">
-        <x:v>Preview 1 child create</x:v>
+        <x:v>Live: lookup 404; không mutation</x:v>
       </x:c>
       <x:c r="E16" s="28" t="str">
-        <x:v>Đạt một phần</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F16" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G16" s="28" t="str">
-        <x:v>Apply và verify parent ID</x:v>
+        <x:v>Giữ guard read-only</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="50" hidden="0" customHeight="1">
       <x:c r="A17" s="28" t="str">
-        <x:v>DRIFT-01</x:v>
+        <x:v>AUTH</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>Manual UI drift</x:v>
+        <x:v>Credential provider</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>IaC không phát hiện thay đổi</x:v>
+        <x:v>Điều kiện chạy</x:v>
       </x:c>
       <x:c r="D17" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Live: thiếu GITHUB_TOKEN trả 401</x:v>
       </x:c>
       <x:c r="E17" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F17" s="28" t="str">
-        <x:v>Team lead</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G17" s="28" t="str">
-        <x:v>Sửa description trên UI</x:v>
+        <x:v>Ghi limitation</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="50" hidden="0" customHeight="1">
       <x:c r="A18" s="28" t="str">
-        <x:v>IMPORT-01</x:v>
+        <x:v>NESTED</x:v>
       </x:c>
       <x:c r="B18" s="28" t="str">
-        <x:v>Import team/membership</x:v>
+        <x:v>Parent/child team</x:v>
       </x:c>
       <x:c r="C18" s="28" t="str">
-        <x:v>Update/replace khi import</x:v>
+        <x:v>Mở rộng ngoài yêu cầu tối thiểu</x:v>
       </x:c>
       <x:c r="D18" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Mock/preview; chưa live</x:v>
       </x:c>
       <x:c r="E18" s="28" t="str">
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F18" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G18" s="28" t="str">
-        <x:v>Dùng team disposable</x:v>
+        <x:v>Không dùng để kết luận task gốc</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="50" hidden="0" customHeight="1">
       <x:c r="A19" s="28" t="str">
-        <x:v>REMOVE-01</x:v>
+        <x:v>DRIFT</x:v>
       </x:c>
       <x:c r="B19" s="28" t="str">
-        <x:v>Remove membership</x:v>
+        <x:v>Manual UI drift</x:v>
       </x:c>
       <x:c r="C19" s="28" t="str">
-        <x:v>Xóa nhầm org member</x:v>
+        <x:v>Mở rộng</x:v>
       </x:c>
       <x:c r="D19" s="28" t="str">
         <x:v>Chưa chạy</x:v>
@@ -2263,21 +2293,21 @@
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F19" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G19" s="28" t="str">
-        <x:v>Plan/show/apply relationship</x:v>
+        <x:v>Chạy sau yêu cầu gốc nếu cần</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="50" hidden="0" customHeight="1">
       <x:c r="A20" s="28" t="str">
-        <x:v>DELETE-01</x:v>
+        <x:v>IMPORT</x:v>
       </x:c>
       <x:c r="B20" s="28" t="str">
-        <x:v>Delete parent</x:v>
+        <x:v>Import team cũ</x:v>
       </x:c>
       <x:c r="C20" s="28" t="str">
-        <x:v>Cascade unmanaged child</x:v>
+        <x:v>Mở rộng</x:v>
       </x:c>
       <x:c r="D20" s="28" t="str">
         <x:v>Chưa chạy</x:v>
@@ -2286,17 +2316,17 @@
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F20" s="28" t="str">
-        <x:v>Org owner</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G20" s="28" t="str">
-        <x:v>Chỉ đánh giá sau inventory</x:v>
+        <x:v>Không chặn kết luận task gốc</x:v>
       </x:c>
     </x:row>
     <x:row r="21"/>
     <x:row r="22"/>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="6" t="str">
-        <x:v>Rủi ro và kiểm soát bắt buộc</x:v>
+        <x:v>Limitation cần ghi trong kết luận</x:v>
       </x:c>
       <x:c r="B23" s="7"/>
       <x:c r="C23" s="7"/>
@@ -2307,163 +2337,163 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="23" t="str">
-        <x:v>Rủi ro</x:v>
+        <x:v>Limitation</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
-        <x:v>Khả năng</x:v>
+        <x:v>Liên quan</x:v>
       </x:c>
       <x:c r="C24" s="23" t="str">
-        <x:v>Tác động</x:v>
+        <x:v>Quan sát</x:v>
       </x:c>
       <x:c r="D24" s="23" t="str">
-        <x:v>Kiểm soát</x:v>
+        <x:v>Cách ghi report</x:v>
       </x:c>
       <x:c r="E24" s="23" t="str">
-        <x:v>Khi nào</x:v>
+        <x:v>Ảnh hưởng</x:v>
       </x:c>
       <x:c r="F24" s="23" t="str">
         <x:v>Owner</x:v>
       </x:c>
       <x:c r="G24" s="23" t="str">
-        <x:v>Mức còn lại</x:v>
+        <x:v>Trạng thái</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="48" hidden="0" customHeight="1">
       <x:c r="A25" s="27" t="str">
-        <x:v>Token quyền rộng</x:v>
+        <x:v>Org Members tách Task 1</x:v>
       </x:c>
       <x:c r="B25" s="27" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>Team membership</x:v>
       </x:c>
       <x:c r="C25" s="27" t="str">
-        <x:v>Cao</x:v>
+        <x:v>Code chỉ lookup read-only</x:v>
       </x:c>
       <x:c r="D25" s="27" t="str">
-        <x:v>GitHub App/PAT ngắn hạn; least privilege; rotation</x:v>
+        <x:v>Không claim invite/update/remove org member</x:v>
       </x:c>
       <x:c r="E25" s="27" t="str">
-        <x:v>Trước Pilot</x:v>
+        <x:v>Cần active member</x:v>
       </x:c>
       <x:c r="F25" s="27" t="str">
-        <x:v>Org owner</x:v>
+        <x:v>Hoàng</x:v>
       </x:c>
       <x:c r="G25" s="27" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>Đang phụ thuộc</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" hidden="0" customHeight="1">
       <x:c r="A26" s="28" t="str">
-        <x:v>State local bị mất/xung đột</x:v>
+        <x:v>Live evidence chưa đủ</x:v>
       </x:c>
       <x:c r="B26" s="28" t="str">
-        <x:v>Cao</x:v>
+        <x:v>Update/delete/role/remove</x:v>
       </x:c>
       <x:c r="C26" s="28" t="str">
-        <x:v>Cao</x:v>
+        <x:v>Phần lớn mới mock hoặc planned</x:v>
       </x:c>
       <x:c r="D26" s="28" t="str">
-        <x:v>Remote backend, encryption, locking, backup</x:v>
+        <x:v>Ghi rõ Chưa chạy</x:v>
       </x:c>
       <x:c r="E26" s="28" t="str">
-        <x:v>Trước Pilot</x:v>
+        <x:v>Chưa kết luận lifecycle</x:v>
       </x:c>
       <x:c r="F26" s="28" t="str">
-        <x:v>Platform lead</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G26" s="28" t="str">
-        <x:v>Thấp</x:v>
+        <x:v>Còn việc</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" hidden="0" customHeight="1">
       <x:c r="A27" s="28" t="str">
-        <x:v>Parent delete cascade</x:v>
+        <x:v>Owner không đại diện user thường</x:v>
       </x:c>
       <x:c r="B27" s="28" t="str">
-        <x:v>Thấp</x:v>
+        <x:v>Team role</x:v>
       </x:c>
       <x:c r="C27" s="28" t="str">
-        <x:v>Cao</x:v>
+        <x:v>Owner luôn được maintainer</x:v>
       </x:c>
       <x:c r="D27" s="28" t="str">
-        <x:v>Inventory child/access; plan review; runbook</x:v>
+        <x:v>Test thêm ordinary member</x:v>
       </x:c>
       <x:c r="E27" s="28" t="str">
-        <x:v>Trước Migration</x:v>
+        <x:v>Chưa đủ role evidence</x:v>
       </x:c>
       <x:c r="F27" s="28" t="str">
-        <x:v>Org owner</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G27" s="28" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>Còn việc</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="48" hidden="0" customHeight="1">
       <x:c r="A28" s="28" t="str">
-        <x:v>Manual drift không reconcile</x:v>
+        <x:v>Membership là additive</x:v>
       </x:c>
       <x:c r="B28" s="28" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>Direct membership</x:v>
       </x:c>
       <x:c r="C28" s="28" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>User ngoài config không tự bị xóa</x:v>
       </x:c>
       <x:c r="D28" s="28" t="str">
-        <x:v>Scheduled plan; break-glass PR trong ngày kế tiếp</x:v>
+        <x:v>Nêu behavior, không claim authoritative list</x:v>
       </x:c>
       <x:c r="E28" s="28" t="str">
-        <x:v>BAU</x:v>
+        <x:v>Giới hạn governance</x:v>
       </x:c>
       <x:c r="F28" s="28" t="str">
-        <x:v>Platform ops</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G28" s="28" t="str">
-        <x:v>Thấp</x:v>
+        <x:v>Đã biết</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="48" hidden="0" customHeight="1">
       <x:c r="A29" s="28" t="str">
-        <x:v>Inherited membership bị hiểu sai</x:v>
+        <x:v>Inherited membership</x:v>
       </x:c>
       <x:c r="B29" s="28" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>Nested team</x:v>
       </x:c>
       <x:c r="C29" s="28" t="str">
-        <x:v>Trung bình</x:v>
+        <x:v>Direct và inherited có thể khác nhau</x:v>
       </x:c>
       <x:c r="D29" s="28" t="str">
-        <x:v>Catalog direct/inherited; test hierarchy</x:v>
+        <x:v>Chỉ claim direct relationship</x:v>
       </x:c>
       <x:c r="E29" s="28" t="str">
-        <x:v>Trước Pilot</x:v>
+        <x:v>Cần kiểm tra riêng</x:v>
       </x:c>
       <x:c r="F29" s="28" t="str">
-        <x:v>Platform</x:v>
+        <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G29" s="28" t="str">
-        <x:v>Thấp</x:v>
+        <x:v>Mở rộng</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="48" hidden="0" customHeight="1">
       <x:c r="A30" s="28" t="str">
-        <x:v>IdP/SCIM conflict</x:v>
+        <x:v>Production controls</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:v>Thấp</x:v>
+        <x:v>Rollout tương lai</x:v>
       </x:c>
       <x:c r="C30" s="28" t="str">
-        <x:v>Cao</x:v>
+        <x:v>Remote state/CI/GitHub App chưa làm</x:v>
       </x:c>
       <x:c r="D30" s="28" t="str">
-        <x:v>Loại synchronized team khỏi Terraform scope</x:v>
+        <x:v>Ghi là recommendation</x:v>
       </x:c>
       <x:c r="E30" s="28" t="str">
-        <x:v>Trước Migration</x:v>
+        <x:v>Ngoài kết luận PoC</x:v>
       </x:c>
       <x:c r="F30" s="28" t="str">
-        <x:v>Identity team</x:v>
+        <x:v>Team lead</x:v>
       </x:c>
       <x:c r="G30" s="28" t="str">
-        <x:v>Thấp</x:v>
+        <x:v>Ngoài phạm vi</x:v>
       </x:c>
     </x:row>
     <x:row r="31"/>
@@ -2518,16 +2548,19 @@
     </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="E9:E20">
-    <x:cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
+    <x:cfRule type="cellIs" dxfId="10" priority="1" operator="equal">
       <x:formula>"Đạt"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="9" priority="2" operator="equal">
+    <x:cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+      <x:formula>"Hoàn tất"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="cellIs" dxfId="12" priority="3" operator="equal">
       <x:formula>"Đạt một phần"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="10" priority="3" operator="equal">
+    <x:cfRule type="cellIs" dxfId="13" priority="4" operator="equal">
       <x:formula>"Chưa chạy"</x:formula>
     </x:cfRule>
-    <x:cfRule type="cellIs" dxfId="11" priority="4" operator="equal">
+    <x:cfRule type="cellIs" dxfId="14" priority="5" operator="equal">
       <x:formula>"Chặn"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
@@ -2538,8 +2571,8 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbbd8d760829d4111"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e504cc6da7148ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcd207b1237041d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82315bf544664470"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete live Task B lifecycle evidence
</commit_message>
<xml_diff>
--- a/outputs/github-org-iac-future-rollout/github-org-iac-future-rollout-vi.xlsx
+++ b/outputs/github-org-iac-future-rollout/github-org-iac-future-rollout-vi.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="Rebdcba8f80f948fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IaC nhưng Manual UI" sheetId="2" r:id="R68d5a35b92ce4b44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lộ trình" sheetId="3" r:id="R31cd41a56bf841fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiểm thử &amp; rủi ro" sheetId="4" r:id="R81ff6aea47154f70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tổng quan" sheetId="1" r:id="Rb659ef4b80c34031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IaC nhưng Manual UI" sheetId="2" r:id="R4b5d28c13b3f489d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lộ trình" sheetId="3" r:id="R75067d7223fa4a0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kiểm thử &amp; rủi ro" sheetId="4" r:id="R7d679c36015c45ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thuật ngữ Provider" sheetId="5" r:id="Ra99f7343e5984157"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -610,7 +611,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R297589f19ea841c5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb7d936540bfa4b75"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -636,14 +637,14 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RolloutRoadmap" displayName="RolloutRoadmap" ref="A4:I9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
-    <x:tableColumn id="1" name="Bước"/>
+    <x:tableColumn id="1" name="Phase"/>
     <x:tableColumn id="2" name="Mục tiêu"/>
     <x:tableColumn id="3" name="Phạm vi"/>
-    <x:tableColumn id="4" name="Bằng chứng cần lưu"/>
-    <x:tableColumn id="5" name="Điều kiện hoàn tất"/>
+    <x:tableColumn id="4" name="Deliverable"/>
+    <x:tableColumn id="5" name="Exit criteria"/>
     <x:tableColumn id="6" name="Owner"/>
-    <x:tableColumn id="7" name="Ước lượng"/>
-    <x:tableColumn id="8" name="Thứ tự"/>
+    <x:tableColumn id="7" name="Tuần"/>
+    <x:tableColumn id="8" name="Bắt đầu"/>
     <x:tableColumn id="9" name="Trạng thái"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -675,6 +676,20 @@
     <x:tableColumn id="5" name="Ảnh hưởng"/>
     <x:tableColumn id="6" name="Owner"/>
     <x:tableColumn id="7" name="Trạng thái"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ProviderTerms" displayName="ProviderTerms" ref="A5:F30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="Thuật ngữ"/>
+    <x:tableColumn id="2" name="Loại"/>
+    <x:tableColumn id="3" name="Nghĩa"/>
+    <x:tableColumn id="4" name="Ví dụ trong PoC"/>
+    <x:tableColumn id="5" name="Khi áp dụng"/>
+    <x:tableColumn id="6" name="Lưu ý"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -959,7 +974,7 @@
       </x:c>
       <x:c r="I5" s="31" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Đạt")</x:f>
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -967,29 +982,29 @@
         <x:v>Đã chứng minh live</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
-        <x:v>Create team + owner direct membership; plan sau apply không đổi</x:v>
+        <x:v>Create/update/delete team; add/role/remove direct membership</x:v>
       </x:c>
       <x:c r="H6" s="28" t="str">
         <x:v>Đạt một phần</x:v>
       </x:c>
       <x:c r="I6" s="32" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Đạt một phần")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="12" t="str">
-        <x:v>Chưa chứng minh live</x:v>
+        <x:v>Trạng thái cuối</x:v>
       </x:c>
       <x:c r="B7" s="13" t="str">
-        <x:v>Update/delete team; add/remove/đổi role member thường</x:v>
+        <x:v>Team đã xóa; Terraform state trống; org members còn nguyên</x:v>
       </x:c>
       <x:c r="H7" s="28" t="str">
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="I7" s="32" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Chưa chạy")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -1004,15 +1019,15 @@
       </x:c>
       <x:c r="I8" s="32" t="n">
         <x:f>COUNTIF('Kiểm thử &amp; rủi ro'!$E$9:$E$20,"Chặn")</x:f>
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A9" s="12" t="str">
         <x:v>Kết luận</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>Khả thi bước đầu; chưa đủ dữ liệu cho toàn bộ lifecycle</x:v>
+        <x:v>Đạt lifecycle Task 2 trong sandbox; chưa đánh giá production</x:v>
       </x:c>
     </x:row>
     <x:row r="10"/>
@@ -1046,104 +1061,104 @@
         <x:v>Quyết định</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="27" t="str">
-        <x:v>Create + convergence</x:v>
+        <x:v>Team lifecycle</x:v>
       </x:c>
       <x:c r="B13" s="27" t="str">
         <x:v>Đạt</x:v>
       </x:c>
       <x:c r="C13" s="27" t="str">
-        <x:v>2 add; follow-up plan = 0</x:v>
+        <x:v>Create/update/delete + convergence</x:v>
       </x:c>
       <x:c r="D13" s="27" t="str">
-        <x:v>Giữ bằng chứng</x:v>
+        <x:v>Giữ Jira evidence</x:v>
       </x:c>
       <x:c r="E13" s="27" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="F13" s="27" t="str">
-        <x:v>Đã chứng minh</x:v>
+        <x:v>Hoàn tất PoC</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="28" t="str">
-        <x:v>Update team</x:v>
+        <x:v>Team membership</x:v>
       </x:c>
       <x:c r="B14" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="C14" s="28" t="str">
-        <x:v>Mới có preview</x:v>
+        <x:v>Add/member→maintainer/remove</x:v>
       </x:c>
       <x:c r="D14" s="28" t="str">
-        <x:v>Apply + UI/state + no-change plan</x:v>
+        <x:v>Org role không đổi</x:v>
       </x:c>
       <x:c r="E14" s="28" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="F14" s="28" t="str">
-        <x:v>Cần chạy</x:v>
+        <x:v>Hoàn tất PoC</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="28" t="str">
-        <x:v>Team membership</x:v>
+        <x:v>Cleanup</x:v>
       </x:c>
       <x:c r="B15" s="28" t="str">
-        <x:v>Đạt một phần</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="C15" s="28" t="str">
-        <x:v>Owner maintainer đạt; user thường chưa thử</x:v>
+        <x:v>Team 404; state empty; final plan 0</x:v>
       </x:c>
       <x:c r="D15" s="28" t="str">
-        <x:v>Add/role/remove với active member</x:v>
+        <x:v>Org members còn active</x:v>
       </x:c>
       <x:c r="E15" s="28" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="F15" s="28" t="str">
-        <x:v>Cần chạy</x:v>
+        <x:v>Hoàn tất PoC</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="28" t="str">
-        <x:v>Delete team</x:v>
+        <x:v>Mở rộng</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>Chưa có live plan/apply</x:v>
+        <x:v>Nested/drift/import chưa live</x:v>
       </x:c>
       <x:c r="D16" s="28" t="str">
-        <x:v>Xóa team disposable an toàn</x:v>
+        <x:v>Chạy nếu pilot cần</x:v>
       </x:c>
       <x:c r="E16" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform</x:v>
       </x:c>
       <x:c r="F16" s="28" t="str">
-        <x:v>Cần chạy</x:v>
+        <x:v>Không chặn task gốc</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="28" t="str">
-        <x:v>Org member lifecycle</x:v>
+        <x:v>Production controls</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>Ngoài phạm vi</x:v>
+        <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>Không có resource mutation trong code</x:v>
+        <x:v>State local; chưa CI/GitHub App</x:v>
       </x:c>
       <x:c r="D17" s="28" t="str">
-        <x:v>Task 1 cung cấp active member</x:v>
+        <x:v>Backend lock + PR + credential</x:v>
       </x:c>
       <x:c r="E17" s="28" t="str">
-        <x:v>Hoàng</x:v>
+        <x:v>Platform lead</x:v>
       </x:c>
       <x:c r="F17" s="28" t="str">
-        <x:v>Phụ thuộc</x:v>
+        <x:v>Chưa production</x:v>
       </x:c>
     </x:row>
     <x:row r="18"/>
@@ -1163,13 +1178,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>Update team trên sandbox</x:v>
+        <x:v>Remote state có locking</x:v>
       </x:c>
       <x:c r="C21" s="11" t="str">
-        <x:v>Name/description/setting; giữ resource identity</x:v>
+        <x:v>Mã hóa, backup và tách workspace/environment</x:v>
       </x:c>
       <x:c r="D21" s="11" t="str">
-        <x:v>Ghi plan, UI/state và no-change plan</x:v>
+        <x:v>Tránh mất state và apply đồng thời</x:v>
       </x:c>
       <x:c r="E21" t="str"/>
       <x:c r="F21" t="str"/>
@@ -1179,13 +1194,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B22" s="11" t="str">
-        <x:v>Nhận active member từ Task 1</x:v>
+        <x:v>Credential chuyên dụng</x:v>
       </x:c>
       <x:c r="C22" s="11" t="str">
-        <x:v>Task 2 không invite hoặc đổi org role</x:v>
+        <x:v>GitHub App hoặc PAT ngắn hạn; least privilege</x:v>
       </x:c>
       <x:c r="D22" s="11" t="str">
-        <x:v>Giữ ranh giới ownership</x:v>
+        <x:v>Không phụ thuộc token cá nhân</x:v>
       </x:c>
       <x:c r="E22" t="str"/>
       <x:c r="F22" t="str"/>
@@ -1195,13 +1210,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B23" s="11" t="str">
-        <x:v>Test team membership</x:v>
+        <x:v>PR + plan review</x:v>
       </x:c>
       <x:c r="C23" s="11" t="str">
-        <x:v>Add, member ↔ maintainer, remove</x:v>
+        <x:v>CI tạo plan; reviewer duyệt destroy/replace</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
-        <x:v>Org membership phải còn nguyên</x:v>
+        <x:v>Có audit trail trước apply</x:v>
       </x:c>
       <x:c r="E23" t="str"/>
       <x:c r="F23" t="str"/>
@@ -1211,13 +1226,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B24" s="11" t="str">
-        <x:v>Test delete team disposable</x:v>
+        <x:v>Pilot import</x:v>
       </x:c>
       <x:c r="C24" s="11" t="str">
-        <x:v>Xem destructive plan trước apply</x:v>
+        <x:v>2–3 team không critical; inventory direct/inherited</x:v>
       </x:c>
       <x:c r="D24" s="11" t="str">
-        <x:v>Xác nhận state và GitHub</x:v>
+        <x:v>Import không tạo diff ngoài dự kiến</x:v>
       </x:c>
       <x:c r="E24" t="str"/>
       <x:c r="F24" t="str"/>
@@ -1227,13 +1242,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B25" s="11" t="str">
-        <x:v>Chốt limitation</x:v>
+        <x:v>Drift và break-glass</x:v>
       </x:c>
       <x:c r="C25" s="11" t="str">
-        <x:v>Ghi behavior thực tế; tách phần mở rộng</x:v>
+        <x:v>Scheduled plan; UI change phải reconcile</x:v>
       </x:c>
       <x:c r="D25" s="11" t="str">
-        <x:v>Đủ bằng chứng cho Task 2</x:v>
+        <x:v>Giữ code là nguồn chuẩn</x:v>
       </x:c>
       <x:c r="E25" t="str"/>
       <x:c r="F25" t="str"/>
@@ -1339,7 +1354,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9974298fc3a64c1d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd798bf7ba73147d3"/>
 </x:worksheet>
 </file>
 
@@ -1622,7 +1637,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref8d42a97c444141"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8abf15a37ae4e38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1647,7 +1662,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
-        <x:v>Các bước hoàn tất Task 2</x:v>
+        <x:v>Cách áp dụng sau PoC</x:v>
       </x:c>
       <x:c r="B1" s="41"/>
       <x:c r="C1" s="41"/>
@@ -1660,7 +1675,7 @@
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Chỉ tính hoàn tất khi có plan/apply, state và kiểm tra thực tế trên GitHub</x:v>
+        <x:v>Triển khai theo từng giai đoạn; PoC đã chứng minh lifecycle tối thiểu trong sandbox</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1674,7 +1689,7 @@
     <x:row r="3"/>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="23" t="str">
-        <x:v>Bước</x:v>
+        <x:v>Phase</x:v>
       </x:c>
       <x:c r="B4" s="23" t="str">
         <x:v>Mục tiêu</x:v>
@@ -1683,19 +1698,19 @@
         <x:v>Phạm vi</x:v>
       </x:c>
       <x:c r="D4" s="23" t="str">
-        <x:v>Bằng chứng cần lưu</x:v>
+        <x:v>Deliverable</x:v>
       </x:c>
       <x:c r="E4" s="23" t="str">
-        <x:v>Điều kiện hoàn tất</x:v>
+        <x:v>Exit criteria</x:v>
       </x:c>
       <x:c r="F4" s="23" t="str">
         <x:v>Owner</x:v>
       </x:c>
       <x:c r="G4" s="23" t="str">
-        <x:v>Ước lượng</x:v>
+        <x:v>Tuần</x:v>
       </x:c>
       <x:c r="H4" s="23" t="str">
-        <x:v>Thứ tự</x:v>
+        <x:v>Bắt đầu</x:v>
       </x:c>
       <x:c r="I4" s="23" t="str">
         <x:v>Trạng thái</x:v>
@@ -1703,22 +1718,22 @@
     </x:row>
     <x:row r="5" ht="56" hidden="0" customHeight="1">
       <x:c r="A5" s="27" t="str">
-        <x:v>0. Baseline</x:v>
+        <x:v>0. PoC</x:v>
       </x:c>
       <x:c r="B5" s="27" t="str">
-        <x:v>Create + convergence</x:v>
+        <x:v>Chứng minh lifecycle</x:v>
       </x:c>
       <x:c r="C5" s="27" t="str">
-        <x:v>1 team + owner membership</x:v>
+        <x:v>Team + direct membership</x:v>
       </x:c>
       <x:c r="D5" s="27" t="str">
-        <x:v>Plan/apply/API/no-change plan</x:v>
+        <x:v>Plan/apply/API/state evidence</x:v>
       </x:c>
       <x:c r="E5" s="27" t="str">
-        <x:v>Đã khớp state và GitHub</x:v>
+        <x:v>Create/update/delete và add/role/remove đạt</x:v>
       </x:c>
       <x:c r="F5" s="27" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform</x:v>
       </x:c>
       <x:c r="G5" s="31" t="n">
         <x:v>1</x:v>
@@ -1732,25 +1747,25 @@
     </x:row>
     <x:row r="6" ht="56" hidden="0" customHeight="1">
       <x:c r="A6" s="28" t="str">
-        <x:v>1. Update team</x:v>
+        <x:v>1. Foundation</x:v>
       </x:c>
       <x:c r="B6" s="28" t="str">
-        <x:v>Kiểm tra update</x:v>
+        <x:v>An toàn state và auth</x:v>
       </x:c>
       <x:c r="C6" s="28" t="str">
-        <x:v>Name/description/setting</x:v>
+        <x:v>Backend lock + credential</x:v>
       </x:c>
       <x:c r="D6" s="28" t="str">
-        <x:v>Plan/apply/UI/state/no-change</x:v>
+        <x:v>Remote state; GitHub App/PAT model</x:v>
       </x:c>
       <x:c r="E6" s="28" t="str">
-        <x:v>Không destroy ngoài dự kiến</x:v>
+        <x:v>Locking và least privilege đạt</x:v>
       </x:c>
       <x:c r="F6" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform lead</x:v>
       </x:c>
       <x:c r="G6" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H6" s="32" t="n">
         <x:f>H5+G5</x:f>
@@ -1762,59 +1777,59 @@
     </x:row>
     <x:row r="7" ht="56" hidden="0" customHeight="1">
       <x:c r="A7" s="28" t="str">
-        <x:v>2. Team membership</x:v>
+        <x:v>2. Workflow</x:v>
       </x:c>
       <x:c r="B7" s="28" t="str">
-        <x:v>Kiểm tra add/role/remove</x:v>
+        <x:v>Review trước apply</x:v>
       </x:c>
       <x:c r="C7" s="28" t="str">
-        <x:v>Active ordinary member</x:v>
+        <x:v>CI + PR</x:v>
       </x:c>
       <x:c r="D7" s="28" t="str">
-        <x:v>Plan/apply/API/state từng bước</x:v>
+        <x:v>Plan artifact; approval; apply job</x:v>
       </x:c>
       <x:c r="E7" s="28" t="str">
-        <x:v>Org member không bị thay đổi</x:v>
+        <x:v>Destroy/replace có reviewer</x:v>
       </x:c>
       <x:c r="F7" s="28" t="str">
-        <x:v>Task 2 + Task 1</x:v>
+        <x:v>Platform</x:v>
       </x:c>
       <x:c r="G7" s="32" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H7" s="32" t="n">
         <x:f>H6+G6</x:f>
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I7" s="28" t="str">
-        <x:v>Chặn</x:v>
+        <x:v>Chưa bắt đầu</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="56" hidden="0" customHeight="1">
       <x:c r="A8" s="28" t="str">
-        <x:v>3. Delete team</x:v>
+        <x:v>3. Pilot</x:v>
       </x:c>
       <x:c r="B8" s="28" t="str">
-        <x:v>Kiểm tra delete</x:v>
+        <x:v>Import scope nhỏ</x:v>
       </x:c>
       <x:c r="C8" s="28" t="str">
-        <x:v>Team disposable</x:v>
+        <x:v>2–3 team không critical</x:v>
       </x:c>
       <x:c r="D8" s="28" t="str">
-        <x:v>Destructive plan đã review</x:v>
+        <x:v>Team catalog + import evidence</x:v>
       </x:c>
       <x:c r="E8" s="28" t="str">
-        <x:v>Remote và state sạch</x:v>
+        <x:v>Hai chu kỳ thay đổi hội tụ</x:v>
       </x:c>
       <x:c r="F8" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform + team lead</x:v>
       </x:c>
       <x:c r="G8" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="H8" s="32" t="n">
         <x:f>H7+G7</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="I8" s="28" t="str">
         <x:v>Chưa bắt đầu</x:v>
@@ -1822,29 +1837,29 @@
     </x:row>
     <x:row r="9" ht="56" hidden="0" customHeight="1">
       <x:c r="A9" s="28" t="str">
-        <x:v>4. Kết luận</x:v>
+        <x:v>4. BAU</x:v>
       </x:c>
       <x:c r="B9" s="28" t="str">
-        <x:v>Chốt limitation</x:v>
+        <x:v>Vận hành định kỳ</x:v>
       </x:c>
       <x:c r="C9" s="28" t="str">
-        <x:v>Đúng yêu cầu gốc</x:v>
+        <x:v>Drift + break-glass</x:v>
       </x:c>
       <x:c r="D9" s="28" t="str">
-        <x:v>Bảng kết quả + behavior</x:v>
+        <x:v>Scheduled plan; runbook; audit</x:v>
       </x:c>
       <x:c r="E9" s="28" t="str">
-        <x:v>Không dùng case dự kiến làm evidence</x:v>
+        <x:v>UI change được reconcile</x:v>
       </x:c>
       <x:c r="F9" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform ops</x:v>
       </x:c>
       <x:c r="G9" s="32" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H9" s="32" t="n">
         <x:f>H8+G8</x:f>
-        <x:v>6</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="I9" s="28" t="str">
         <x:v>Chưa bắt đầu</x:v>
@@ -1878,46 +1893,46 @@
     </x:row>
     <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="27" t="str">
-        <x:v>Active ordinary member</x:v>
+        <x:v>Ranh giới ownership</x:v>
       </x:c>
       <x:c r="B14" s="27" t="str">
-        <x:v>Cần test add/role/remove team membership</x:v>
+        <x:v>Org Members và Org Teams có lifecycle khác nhau</x:v>
       </x:c>
       <x:c r="C14" s="27" t="str">
-        <x:v>Nhận từ Task 1</x:v>
+        <x:v>Tách state/module hoặc owner rõ</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" hidden="0" customHeight="1">
       <x:c r="A15" s="28" t="str">
-        <x:v>Plan trước destructive apply</x:v>
+        <x:v>Remote state + locking</x:v>
       </x:c>
       <x:c r="B15" s="28" t="str">
-        <x:v>Delete/remove là yêu cầu gốc nhưng có tác động thật</x:v>
+        <x:v>Nhiều admin không được apply cùng state</x:v>
       </x:c>
       <x:c r="C15" s="28" t="str">
-        <x:v>Bắt buộc</x:v>
+        <x:v>Bắt buộc trước pilot</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" hidden="0" customHeight="1">
       <x:c r="A16" s="28" t="str">
-        <x:v>UI/API + state + no-change plan</x:v>
+        <x:v>Plan trước destructive apply</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
-        <x:v>Một apply thành công chưa đủ chứng minh hội tụ</x:v>
+        <x:v>Team delete có thể ảnh hưởng access và child team</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>Bắt buộc mỗi flow</x:v>
+        <x:v>Bắt buộc mọi environment</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="28" t="str">
-        <x:v>Tách planned và verified</x:v>
+        <x:v>Inventory direct/inherited</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>Tránh trình bày kỳ vọng như kết quả thực tế</x:v>
+        <x:v>Nested team làm membership khó đọc</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>Bắt buộc trong report</x:v>
+        <x:v>Bắt buộc trước import</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1945,7 +1960,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e4796a130dd4252"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3596157278b84e8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1968,7 +1983,7 @@
   <x:sheetData>
     <x:row r="1" ht="24" hidden="0" customHeight="1">
       <x:c r="A1" s="40" t="str">
-        <x:v>Bằng chứng và phần việc còn lại</x:v>
+        <x:v>Bằng chứng và giới hạn</x:v>
       </x:c>
       <x:c r="B1" s="41"/>
       <x:c r="C1" s="41"/>
@@ -1979,7 +1994,7 @@
     </x:row>
     <x:row r="2" ht="24" hidden="0" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Live = đã plan/apply và đối chiếu GitHub/state; mock hoặc preview không thay thế live evidence</x:v>
+        <x:v>Task gốc đã hoàn tất live; các phần mở rộng và production controls vẫn cần đánh giá riêng</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -2006,19 +2021,19 @@
     <x:row r="5" ht="16.799999237060547" hidden="0" customHeight="1">
       <x:c r="A5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Đạt")</x:f>
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="B5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Đạt một phần")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Chưa chạy")</x:f>
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D5" s="39" t="n">
         <x:f>COUNTIF($E$9:$E$20,"Chặn")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="6"/>
@@ -2071,16 +2086,16 @@
     </x:row>
     <x:row r="10" ht="50" hidden="0" customHeight="1">
       <x:c r="A10" s="28" t="str">
-        <x:v>CONVERGE</x:v>
+        <x:v>TEAM-UPDATE</x:v>
       </x:c>
       <x:c r="B10" s="28" t="str">
-        <x:v>Plan sau apply</x:v>
+        <x:v>Update team</x:v>
       </x:c>
       <x:c r="C10" s="28" t="str">
-        <x:v>Xác minh state</x:v>
+        <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D10" s="28" t="str">
-        <x:v>Live: exit 0, no changes</x:v>
+        <x:v>Live: update in-place; giữ ID 19806617</x:v>
       </x:c>
       <x:c r="E10" s="28" t="str">
         <x:v>Đạt</x:v>
@@ -2089,136 +2104,136 @@
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G10" s="28" t="str">
-        <x:v>Lặp lại sau mỗi flow</x:v>
+        <x:v>Giữ evidence</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="50" hidden="0" customHeight="1">
       <x:c r="A11" s="28" t="str">
-        <x:v>TEAM-UPDATE</x:v>
+        <x:v>TEAM-DELETE</x:v>
       </x:c>
       <x:c r="B11" s="28" t="str">
-        <x:v>Update team</x:v>
+        <x:v>Delete team</x:v>
       </x:c>
       <x:c r="C11" s="28" t="str">
         <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D11" s="28" t="str">
-        <x:v>Chỉ có preview; chưa apply</x:v>
+        <x:v>Live: plan review; team 404; state empty</x:v>
       </x:c>
       <x:c r="E11" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F11" s="28" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G11" s="28" t="str">
-        <x:v>Apply và verify</x:v>
+        <x:v>Giữ destructive gate</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="50" hidden="0" customHeight="1">
       <x:c r="A12" s="28" t="str">
-        <x:v>TEAM-DELETE</x:v>
+        <x:v>MEMBER-ADD</x:v>
       </x:c>
       <x:c r="B12" s="28" t="str">
-        <x:v>Delete team</x:v>
+        <x:v>Add member vào team</x:v>
       </x:c>
       <x:c r="C12" s="28" t="str">
         <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D12" s="28" t="str">
-        <x:v>Chưa có live plan/apply</x:v>
+        <x:v>Live: phuc776 active/member</x:v>
       </x:c>
       <x:c r="E12" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F12" s="28" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G12" s="28" t="str">
-        <x:v>Dùng team disposable</x:v>
+        <x:v>Giữ active-member guard</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="50" hidden="0" customHeight="1">
       <x:c r="A13" s="28" t="str">
-        <x:v>MEMBER-ADD</x:v>
+        <x:v>MEMBER-ROLE</x:v>
       </x:c>
       <x:c r="B13" s="28" t="str">
-        <x:v>Add member vào team</x:v>
+        <x:v>Đổi team role</x:v>
       </x:c>
       <x:c r="C13" s="28" t="str">
         <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D13" s="28" t="str">
-        <x:v>Owner đã được add; user thường chưa thử</x:v>
+        <x:v>Live: member → maintainer in-place</x:v>
       </x:c>
       <x:c r="E13" s="28" t="str">
-        <x:v>Đạt một phần</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F13" s="28" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G13" s="28" t="str">
-        <x:v>Cần active ordinary member</x:v>
+        <x:v>Org role không đổi</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="50" hidden="0" customHeight="1">
       <x:c r="A14" s="28" t="str">
-        <x:v>MEMBER-ROLE</x:v>
+        <x:v>MEMBER-REMOVE</x:v>
       </x:c>
       <x:c r="B14" s="28" t="str">
-        <x:v>Đổi team role</x:v>
+        <x:v>Remove member khỏi team</x:v>
       </x:c>
       <x:c r="C14" s="28" t="str">
         <x:v>Yêu cầu gốc</x:v>
       </x:c>
       <x:c r="D14" s="28" t="str">
-        <x:v>Mock đạt; chưa có active user thường</x:v>
+        <x:v>Live: relationship 404; org active/member</x:v>
       </x:c>
       <x:c r="E14" s="28" t="str">
-        <x:v>Chặn</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F14" s="28" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G14" s="28" t="str">
-        <x:v>Phụ thuộc Task 1</x:v>
+        <x:v>Giữ boundary</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="50" hidden="0" customHeight="1">
       <x:c r="A15" s="28" t="str">
-        <x:v>MEMBER-REMOVE</x:v>
+        <x:v>CONVERGE</x:v>
       </x:c>
       <x:c r="B15" s="28" t="str">
-        <x:v>Remove member khỏi team</x:v>
+        <x:v>Plan sau apply</x:v>
       </x:c>
       <x:c r="C15" s="28" t="str">
-        <x:v>Yêu cầu gốc</x:v>
+        <x:v>Xác minh state</x:v>
       </x:c>
       <x:c r="D15" s="28" t="str">
-        <x:v>Chưa có active user thường</x:v>
+        <x:v>Live: exit 0 sau mỗi flow</x:v>
       </x:c>
       <x:c r="E15" s="28" t="str">
-        <x:v>Chặn</x:v>
+        <x:v>Đạt</x:v>
       </x:c>
       <x:c r="F15" s="28" t="str">
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G15" s="28" t="str">
-        <x:v>Phụ thuộc Task 1</x:v>
+        <x:v>Bắt buộc trong pipeline</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="50" hidden="0" customHeight="1">
       <x:c r="A16" s="28" t="str">
-        <x:v>OUTSIDER</x:v>
+        <x:v>BOUNDARY</x:v>
       </x:c>
       <x:c r="B16" s="28" t="str">
-        <x:v>User chưa thuộc org</x:v>
+        <x:v>Org member không bị xóa</x:v>
       </x:c>
       <x:c r="C16" s="28" t="str">
-        <x:v>Boundary Task 1/2</x:v>
+        <x:v>Task 1/2</x:v>
       </x:c>
       <x:c r="D16" s="28" t="str">
-        <x:v>Live: lookup 404; không mutation</x:v>
+        <x:v>Live: cả hai user còn active sau cleanup</x:v>
       </x:c>
       <x:c r="E16" s="28" t="str">
         <x:v>Đạt</x:v>
@@ -2227,61 +2242,61 @@
         <x:v>Task 2</x:v>
       </x:c>
       <x:c r="G16" s="28" t="str">
-        <x:v>Giữ guard read-only</x:v>
+        <x:v>Tách ownership</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="50" hidden="0" customHeight="1">
       <x:c r="A17" s="28" t="str">
-        <x:v>AUTH</x:v>
+        <x:v>NESTED</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>Credential provider</x:v>
+        <x:v>Parent/child team</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>Điều kiện chạy</x:v>
+        <x:v>Mở rộng</x:v>
       </x:c>
       <x:c r="D17" s="28" t="str">
-        <x:v>Live: thiếu GITHUB_TOKEN trả 401</x:v>
+        <x:v>Mock/preview; chưa live</x:v>
       </x:c>
       <x:c r="E17" s="28" t="str">
-        <x:v>Đạt</x:v>
+        <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F17" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform</x:v>
       </x:c>
       <x:c r="G17" s="28" t="str">
-        <x:v>Ghi limitation</x:v>
+        <x:v>Đánh giá trước pilot</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="50" hidden="0" customHeight="1">
       <x:c r="A18" s="28" t="str">
-        <x:v>NESTED</x:v>
+        <x:v>DRIFT</x:v>
       </x:c>
       <x:c r="B18" s="28" t="str">
-        <x:v>Parent/child team</x:v>
+        <x:v>Manual UI drift</x:v>
       </x:c>
       <x:c r="C18" s="28" t="str">
-        <x:v>Mở rộng ngoài yêu cầu tối thiểu</x:v>
+        <x:v>Mở rộng</x:v>
       </x:c>
       <x:c r="D18" s="28" t="str">
-        <x:v>Mock/preview; chưa live</x:v>
+        <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="E18" s="28" t="str">
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F18" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform</x:v>
       </x:c>
       <x:c r="G18" s="28" t="str">
-        <x:v>Không dùng để kết luận task gốc</x:v>
+        <x:v>Scheduled plan</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="50" hidden="0" customHeight="1">
       <x:c r="A19" s="28" t="str">
-        <x:v>DRIFT</x:v>
+        <x:v>IMPORT</x:v>
       </x:c>
       <x:c r="B19" s="28" t="str">
-        <x:v>Manual UI drift</x:v>
+        <x:v>Import team cũ</x:v>
       </x:c>
       <x:c r="C19" s="28" t="str">
         <x:v>Mở rộng</x:v>
@@ -2293,33 +2308,33 @@
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F19" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform</x:v>
       </x:c>
       <x:c r="G19" s="28" t="str">
-        <x:v>Chạy sau yêu cầu gốc nếu cần</x:v>
+        <x:v>Pilot team disposable</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="50" hidden="0" customHeight="1">
       <x:c r="A20" s="28" t="str">
-        <x:v>IMPORT</x:v>
+        <x:v>PROD</x:v>
       </x:c>
       <x:c r="B20" s="28" t="str">
-        <x:v>Import team cũ</x:v>
+        <x:v>State/auth/CI</x:v>
       </x:c>
       <x:c r="C20" s="28" t="str">
-        <x:v>Mở rộng</x:v>
+        <x:v>Production</x:v>
       </x:c>
       <x:c r="D20" s="28" t="str">
-        <x:v>Chưa chạy</x:v>
+        <x:v>State local; chưa pipeline/GitHub App</x:v>
       </x:c>
       <x:c r="E20" s="28" t="str">
         <x:v>Chưa chạy</x:v>
       </x:c>
       <x:c r="F20" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform lead</x:v>
       </x:c>
       <x:c r="G20" s="28" t="str">
-        <x:v>Không chặn kết luận task gốc</x:v>
+        <x:v>Foundation phase</x:v>
       </x:c>
     </x:row>
     <x:row r="21"/>
@@ -2363,42 +2378,42 @@
         <x:v>Org Members tách Task 1</x:v>
       </x:c>
       <x:c r="B25" s="27" t="str">
-        <x:v>Team membership</x:v>
+        <x:v>Invitation/org role/remove</x:v>
       </x:c>
       <x:c r="C25" s="27" t="str">
-        <x:v>Code chỉ lookup read-only</x:v>
+        <x:v>Task 2 chỉ lookup read-only</x:v>
       </x:c>
       <x:c r="D25" s="27" t="str">
-        <x:v>Không claim invite/update/remove org member</x:v>
+        <x:v>Tách state và ownership</x:v>
       </x:c>
       <x:c r="E25" s="27" t="str">
-        <x:v>Cần active member</x:v>
+        <x:v>Tránh xóa nhầm org member</x:v>
       </x:c>
       <x:c r="F25" s="27" t="str">
-        <x:v>Hoàng</x:v>
+        <x:v>Org admin</x:v>
       </x:c>
       <x:c r="G25" s="27" t="str">
-        <x:v>Đang phụ thuộc</x:v>
+        <x:v>Đã giữ boundary</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" hidden="0" customHeight="1">
       <x:c r="A26" s="28" t="str">
-        <x:v>Live evidence chưa đủ</x:v>
+        <x:v>State local</x:v>
       </x:c>
       <x:c r="B26" s="28" t="str">
-        <x:v>Update/delete/role/remove</x:v>
+        <x:v>Nhiều admin</x:v>
       </x:c>
       <x:c r="C26" s="28" t="str">
-        <x:v>Phần lớn mới mock hoặc planned</x:v>
+        <x:v>Không có locking hoặc shared backup</x:v>
       </x:c>
       <x:c r="D26" s="28" t="str">
-        <x:v>Ghi rõ Chưa chạy</x:v>
+        <x:v>Remote backend trước pilot</x:v>
       </x:c>
       <x:c r="E26" s="28" t="str">
-        <x:v>Chưa kết luận lifecycle</x:v>
+        <x:v>Chưa production</x:v>
       </x:c>
       <x:c r="F26" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Platform lead</x:v>
       </x:c>
       <x:c r="G26" s="28" t="str">
         <x:v>Còn việc</x:v>
@@ -2406,22 +2421,22 @@
     </x:row>
     <x:row r="27" ht="48" hidden="0" customHeight="1">
       <x:c r="A27" s="28" t="str">
-        <x:v>Owner không đại diện user thường</x:v>
+        <x:v>Credential cá nhân</x:v>
       </x:c>
       <x:c r="B27" s="28" t="str">
-        <x:v>Team role</x:v>
+        <x:v>Authentication</x:v>
       </x:c>
       <x:c r="C27" s="28" t="str">
-        <x:v>Owner luôn được maintainer</x:v>
+        <x:v>PoC dùng credential process-local</x:v>
       </x:c>
       <x:c r="D27" s="28" t="str">
-        <x:v>Test thêm ordinary member</x:v>
+        <x:v>GitHub App/PAT chuyên dụng</x:v>
       </x:c>
       <x:c r="E27" s="28" t="str">
-        <x:v>Chưa đủ role evidence</x:v>
+        <x:v>Chưa production</x:v>
       </x:c>
       <x:c r="F27" s="28" t="str">
-        <x:v>Task 2</x:v>
+        <x:v>Org admin</x:v>
       </x:c>
       <x:c r="G27" s="28" t="str">
         <x:v>Còn việc</x:v>
@@ -2475,25 +2490,25 @@
     </x:row>
     <x:row r="30" ht="48" hidden="0" customHeight="1">
       <x:c r="A30" s="28" t="str">
-        <x:v>Production controls</x:v>
+        <x:v>IdP-synchronized team</x:v>
       </x:c>
       <x:c r="B30" s="28" t="str">
-        <x:v>Rollout tương lai</x:v>
+        <x:v>Team membership</x:v>
       </x:c>
       <x:c r="C30" s="28" t="str">
-        <x:v>Remote state/CI/GitHub App chưa làm</x:v>
+        <x:v>GitHub API chặn thay đổi trực tiếp</x:v>
       </x:c>
       <x:c r="D30" s="28" t="str">
-        <x:v>Ghi là recommendation</x:v>
+        <x:v>Loại khỏi scope hoặc quản lý ở IdP</x:v>
       </x:c>
       <x:c r="E30" s="28" t="str">
-        <x:v>Ngoài kết luận PoC</x:v>
+        <x:v>Cần policy riêng</x:v>
       </x:c>
       <x:c r="F30" s="28" t="str">
-        <x:v>Team lead</x:v>
+        <x:v>Identity team</x:v>
       </x:c>
       <x:c r="G30" s="28" t="str">
-        <x:v>Ngoài phạm vi</x:v>
+        <x:v>Mở rộng</x:v>
       </x:c>
     </x:row>
     <x:row r="31"/>
@@ -2571,8 +2586,624 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcd207b1237041d2"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82315bf544664470"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc07c9321df0e4322"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rade040bbccf44585"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF8064A2"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A1" s="40" t="str">
+        <x:v>Thuật ngữ Terraform và GitHub Provider</x:v>
+      </x:c>
+      <x:c r="B1" s="41"/>
+      <x:c r="C1" s="41"/>
+      <x:c r="D1" s="41"/>
+      <x:c r="E1" s="41"/>
+      <x:c r="F1" s="41"/>
+    </x:row>
+    <x:row r="2" ht="24" hidden="0" customHeight="1">
+      <x:c r="A2" s="3" t="str">
+        <x:v>Các khái niệm cần biết khi đọc plan, state và thiết kế cách quản lý organization bằng IaC</x:v>
+      </x:c>
+      <x:c r="B2" s="3"/>
+      <x:c r="C2" s="3"/>
+      <x:c r="D2" s="3"/>
+      <x:c r="E2" s="3"/>
+      <x:c r="F2" s="3"/>
+    </x:row>
+    <x:row r="3"/>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>Từ điển áp dụng</x:v>
+      </x:c>
+      <x:c r="B4" s="7"/>
+      <x:c r="C4" s="7"/>
+      <x:c r="D4" s="7"/>
+      <x:c r="E4" s="7"/>
+      <x:c r="F4" s="8"/>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>Thuật ngữ</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="str">
+        <x:v>Loại</x:v>
+      </x:c>
+      <x:c r="C5" s="23" t="str">
+        <x:v>Nghĩa</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>Ví dụ trong PoC</x:v>
+      </x:c>
+      <x:c r="E5" s="23" t="str">
+        <x:v>Khi áp dụng</x:v>
+      </x:c>
+      <x:c r="F5" s="23" t="str">
+        <x:v>Lưu ý</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="48" hidden="0" customHeight="1">
+      <x:c r="A6" s="27" t="str">
+        <x:v>Provider</x:v>
+      </x:c>
+      <x:c r="B6" s="27" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C6" s="27" t="str">
+        <x:v>Plugin kết nối Terraform với GitHub API</x:v>
+      </x:c>
+      <x:c r="D6" s="27" t="str">
+        <x:v>integrations/github 6.13.0</x:v>
+      </x:c>
+      <x:c r="E6" s="27" t="str">
+        <x:v>Mọi resource/data GitHub</x:v>
+      </x:c>
+      <x:c r="F6" s="27" t="str">
+        <x:v>Pin version và lock file</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="48" hidden="0" customHeight="1">
+      <x:c r="A7" s="28" t="str">
+        <x:v>Resource</x:v>
+      </x:c>
+      <x:c r="B7" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C7" s="28" t="str">
+        <x:v>Đối tượng Terraform tạo, cập nhật hoặc xóa</x:v>
+      </x:c>
+      <x:c r="D7" s="28" t="str">
+        <x:v>github_team</x:v>
+      </x:c>
+      <x:c r="E7" s="28" t="str">
+        <x:v>Khi IaC sở hữu lifecycle</x:v>
+      </x:c>
+      <x:c r="F7" s="28" t="str">
+        <x:v>Bỏ khỏi config thường tạo destroy</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="48" hidden="0" customHeight="1">
+      <x:c r="A8" s="28" t="str">
+        <x:v>Data source</x:v>
+      </x:c>
+      <x:c r="B8" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C8" s="28" t="str">
+        <x:v>Chỉ đọc dữ liệu có sẵn</x:v>
+      </x:c>
+      <x:c r="D8" s="28" t="str">
+        <x:v>data.github_membership.existing</x:v>
+      </x:c>
+      <x:c r="E8" s="28" t="str">
+        <x:v>Kiểm tra prerequisite</x:v>
+      </x:c>
+      <x:c r="F8" s="28" t="str">
+        <x:v>Không gửi invitation trong PoC</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="48" hidden="0" customHeight="1">
+      <x:c r="A9" s="28" t="str">
+        <x:v>Configuration</x:v>
+      </x:c>
+      <x:c r="B9" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C9" s="28" t="str">
+        <x:v>Code mô tả trạng thái mong muốn</x:v>
+      </x:c>
+      <x:c r="D9" s="28" t="str">
+        <x:v>teams map trong tfvars</x:v>
+      </x:c>
+      <x:c r="E9" s="28" t="str">
+        <x:v>Review qua Git</x:v>
+      </x:c>
+      <x:c r="F9" s="28" t="str">
+        <x:v>Không chứa token/state</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="48" hidden="0" customHeight="1">
+      <x:c r="A10" s="28" t="str">
+        <x:v>Desired state</x:v>
+      </x:c>
+      <x:c r="B10" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C10" s="28" t="str">
+        <x:v>Trạng thái đích khai báo trong code</x:v>
+      </x:c>
+      <x:c r="D10" s="28" t="str">
+        <x:v>Team name, role, privacy</x:v>
+      </x:c>
+      <x:c r="E10" s="28" t="str">
+        <x:v>Plan so sánh với remote</x:v>
+      </x:c>
+      <x:c r="F10" s="28" t="str">
+        <x:v>Khác remote sẽ tạo diff</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="48" hidden="0" customHeight="1">
+      <x:c r="A11" s="28" t="str">
+        <x:v>State</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C11" s="28" t="str">
+        <x:v>Ánh xạ resource address với object GitHub</x:v>
+      </x:c>
+      <x:c r="D11" s="28" t="str">
+        <x:v>Team ID 19806617</x:v>
+      </x:c>
+      <x:c r="E11" s="28" t="str">
+        <x:v>Refresh, update, delete</x:v>
+      </x:c>
+      <x:c r="F11" s="28" t="str">
+        <x:v>Có dữ liệu nhạy cảm; cần bảo vệ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="48" hidden="0" customHeight="1">
+      <x:c r="A12" s="28" t="str">
+        <x:v>Backend</x:v>
+      </x:c>
+      <x:c r="B12" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C12" s="28" t="str">
+        <x:v>Nơi lưu state</x:v>
+      </x:c>
+      <x:c r="D12" s="28" t="str">
+        <x:v>PoC dùng local state</x:v>
+      </x:c>
+      <x:c r="E12" s="28" t="str">
+        <x:v>Production dùng remote backend</x:v>
+      </x:c>
+      <x:c r="F12" s="28" t="str">
+        <x:v>Cần encryption, backup, access control</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="48" hidden="0" customHeight="1">
+      <x:c r="A13" s="28" t="str">
+        <x:v>State locking</x:v>
+      </x:c>
+      <x:c r="B13" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C13" s="28" t="str">
+        <x:v>Khóa state khi một run đang ghi</x:v>
+      </x:c>
+      <x:c r="D13" s="28" t="str">
+        <x:v>PoC chưa có</x:v>
+      </x:c>
+      <x:c r="E13" s="28" t="str">
+        <x:v>Nhiều admin hoặc CI</x:v>
+      </x:c>
+      <x:c r="F13" s="28" t="str">
+        <x:v>Ngăn apply đồng thời</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="48" hidden="0" customHeight="1">
+      <x:c r="A14" s="28" t="str">
+        <x:v>Plan</x:v>
+      </x:c>
+      <x:c r="B14" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C14" s="28" t="str">
+        <x:v>Preview diff trước mutation</x:v>
+      </x:c>
+      <x:c r="D14" s="28" t="str">
+        <x:v>0 add / 1 change / 0 destroy</x:v>
+      </x:c>
+      <x:c r="E14" s="28" t="str">
+        <x:v>Bắt buộc trước apply</x:v>
+      </x:c>
+      <x:c r="F14" s="28" t="str">
+        <x:v>Saved plan có thể stale</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="48" hidden="0" customHeight="1">
+      <x:c r="A15" s="28" t="str">
+        <x:v>Apply</x:v>
+      </x:c>
+      <x:c r="B15" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C15" s="28" t="str">
+        <x:v>Thực thi plan lên GitHub</x:v>
+      </x:c>
+      <x:c r="D15" s="28" t="str">
+        <x:v>Update team in-place</x:v>
+      </x:c>
+      <x:c r="E15" s="28" t="str">
+        <x:v>Sau review</x:v>
+      </x:c>
+      <x:c r="F15" s="28" t="str">
+        <x:v>Sau apply phải verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="48" hidden="0" customHeight="1">
+      <x:c r="A16" s="28" t="str">
+        <x:v>Refresh</x:v>
+      </x:c>
+      <x:c r="B16" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C16" s="28" t="str">
+        <x:v>Đọc remote để cập nhật góc nhìn của state</x:v>
+      </x:c>
+      <x:c r="D16" s="28" t="str">
+        <x:v>Plan đọc team/membership</x:v>
+      </x:c>
+      <x:c r="E16" s="28" t="str">
+        <x:v>Trước khi tính diff</x:v>
+      </x:c>
+      <x:c r="F16" s="28" t="str">
+        <x:v>Cần credential hợp lệ</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="48" hidden="0" customHeight="1">
+      <x:c r="A17" s="28" t="str">
+        <x:v>Drift</x:v>
+      </x:c>
+      <x:c r="B17" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C17" s="28" t="str">
+        <x:v>Remote bị sửa khác code</x:v>
+      </x:c>
+      <x:c r="D17" s="28" t="str">
+        <x:v>Sửa description bằng UI</x:v>
+      </x:c>
+      <x:c r="E17" s="28" t="str">
+        <x:v>Scheduled plan phát hiện</x:v>
+      </x:c>
+      <x:c r="F17" s="28" t="str">
+        <x:v>Chọn restore code hoặc cập nhật code</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="48" hidden="0" customHeight="1">
+      <x:c r="A18" s="28" t="str">
+        <x:v>Import</x:v>
+      </x:c>
+      <x:c r="B18" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C18" s="28" t="str">
+        <x:v>Đưa object có sẵn vào state</x:v>
+      </x:c>
+      <x:c r="D18" s="28" t="str">
+        <x:v>Import bằng numeric team ID</x:v>
+      </x:c>
+      <x:c r="E18" s="28" t="str">
+        <x:v>Migration team hiện hữu</x:v>
+      </x:c>
+      <x:c r="F18" s="28" t="str">
+        <x:v>Config phải khớp trước apply</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="48" hidden="0" customHeight="1">
+      <x:c r="A19" s="28" t="str">
+        <x:v>for_each key</x:v>
+      </x:c>
+      <x:c r="B19" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C19" s="28" t="str">
+        <x:v>Key ổn định tạo identity trong state</x:v>
+      </x:c>
+      <x:c r="D19" s="28" t="str">
+        <x:v>devops</x:v>
+      </x:c>
+      <x:c r="E19" s="28" t="str">
+        <x:v>Quản lý nhiều team</x:v>
+      </x:c>
+      <x:c r="F19" s="28" t="str">
+        <x:v>Đổi key có thể destroy/create</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="48" hidden="0" customHeight="1">
+      <x:c r="A20" s="28" t="str">
+        <x:v>Resource address</x:v>
+      </x:c>
+      <x:c r="B20" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C20" s="28" t="str">
+        <x:v>Địa chỉ duy nhất của instance trong state</x:v>
+      </x:c>
+      <x:c r="D20" s="28" t="str">
+        <x:v>github_team.root["devops"]</x:v>
+      </x:c>
+      <x:c r="E20" s="28" t="str">
+        <x:v>Plan, import, state commands</x:v>
+      </x:c>
+      <x:c r="F20" s="28" t="str">
+        <x:v>Phải quote đúng trên shell</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" hidden="0" customHeight="1">
+      <x:c r="A21" s="28" t="str">
+        <x:v>Dependency</x:v>
+      </x:c>
+      <x:c r="B21" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C21" s="28" t="str">
+        <x:v>Quan hệ xác định thứ tự xử lý</x:v>
+      </x:c>
+      <x:c r="D21" s="28" t="str">
+        <x:v>Membership phụ thuộc team ID</x:v>
+      </x:c>
+      <x:c r="E21" s="28" t="str">
+        <x:v>Parent/child và memberships</x:v>
+      </x:c>
+      <x:c r="F21" s="28" t="str">
+        <x:v>Tránh cycle</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" hidden="0" customHeight="1">
+      <x:c r="A22" s="28" t="str">
+        <x:v>Output</x:v>
+      </x:c>
+      <x:c r="B22" s="28" t="str">
+        <x:v>Terraform</x:v>
+      </x:c>
+      <x:c r="C22" s="28" t="str">
+        <x:v>Giá trị xuất ra sau plan/apply</x:v>
+      </x:c>
+      <x:c r="D22" s="28" t="str">
+        <x:v>team ID, slug, URL</x:v>
+      </x:c>
+      <x:c r="E22" s="28" t="str">
+        <x:v>Verification và integration</x:v>
+      </x:c>
+      <x:c r="F22" s="28" t="str">
+        <x:v>Không output secret</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="48" hidden="0" customHeight="1">
+      <x:c r="A23" s="28" t="str">
+        <x:v>github_team</x:v>
+      </x:c>
+      <x:c r="B23" s="28" t="str">
+        <x:v>GitHub Provider</x:v>
+      </x:c>
+      <x:c r="C23" s="28" t="str">
+        <x:v>Quản lý team properties và hierarchy</x:v>
+      </x:c>
+      <x:c r="D23" s="28" t="str">
+        <x:v>poc-infra-maintainers</x:v>
+      </x:c>
+      <x:c r="E23" s="28" t="str">
+        <x:v>Create/update/delete team</x:v>
+      </x:c>
+      <x:c r="F23" s="28" t="str">
+        <x:v>Delete có thể ảnh hưởng access/child</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="48" hidden="0" customHeight="1">
+      <x:c r="A24" s="28" t="str">
+        <x:v>github_team_membership</x:v>
+      </x:c>
+      <x:c r="B24" s="28" t="str">
+        <x:v>GitHub Provider</x:v>
+      </x:c>
+      <x:c r="C24" s="28" t="str">
+        <x:v>Quản lý một direct team/user relationship</x:v>
+      </x:c>
+      <x:c r="D24" s="28" t="str">
+        <x:v>phuc776: member → maintainer</x:v>
+      </x:c>
+      <x:c r="E24" s="28" t="str">
+        <x:v>Add/role/remove team member</x:v>
+      </x:c>
+      <x:c r="F24" s="28" t="str">
+        <x:v>Không đại diện inherited membership</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="48" hidden="0" customHeight="1">
+      <x:c r="A25" s="28" t="str">
+        <x:v>github_membership</x:v>
+      </x:c>
+      <x:c r="B25" s="28" t="str">
+        <x:v>GitHub Provider</x:v>
+      </x:c>
+      <x:c r="C25" s="28" t="str">
+        <x:v>Quản lý organization member và gửi invitation</x:v>
+      </x:c>
+      <x:c r="D25" s="28" t="str">
+        <x:v>Thuộc Task Org Members</x:v>
+      </x:c>
+      <x:c r="E25" s="28" t="str">
+        <x:v>Invite/update org role/remove</x:v>
+      </x:c>
+      <x:c r="F25" s="28" t="str">
+        <x:v>Destroy có thể remove user khỏi org</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="48" hidden="0" customHeight="1">
+      <x:c r="A26" s="28" t="str">
+        <x:v>Implicit team invitation</x:v>
+      </x:c>
+      <x:c r="B26" s="28" t="str">
+        <x:v>GitHub API</x:v>
+      </x:c>
+      <x:c r="C26" s="28" t="str">
+        <x:v>Owner thêm non-member vào team sẽ gửi org invitation</x:v>
+      </x:c>
+      <x:c r="D26" s="28" t="str">
+        <x:v>PoC chủ động chặn bằng active lookup</x:v>
+      </x:c>
+      <x:c r="E26" s="28" t="str">
+        <x:v>Chỉ khi muốn gộp invite + team</x:v>
+      </x:c>
+      <x:c r="F26" s="28" t="str">
+        <x:v>Khuyến nghị tách Task Org Members</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="48" hidden="0" customHeight="1">
+      <x:c r="A27" s="28" t="str">
+        <x:v>Role</x:v>
+      </x:c>
+      <x:c r="B27" s="28" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="C27" s="28" t="str">
+        <x:v>Quyền ở org hoặc team</x:v>
+      </x:c>
+      <x:c r="D27" s="28" t="str">
+        <x:v>Org member; team maintainer</x:v>
+      </x:c>
+      <x:c r="E27" s="28" t="str">
+        <x:v>Phân quyền</x:v>
+      </x:c>
+      <x:c r="F27" s="28" t="str">
+        <x:v>Org admin khác team maintainer</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="48" hidden="0" customHeight="1">
+      <x:c r="A28" s="28" t="str">
+        <x:v>active / pending</x:v>
+      </x:c>
+      <x:c r="B28" s="28" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="C28" s="28" t="str">
+        <x:v>Trạng thái organization/team membership</x:v>
+      </x:c>
+      <x:c r="D28" s="28" t="str">
+        <x:v>phuc776 active trước add</x:v>
+      </x:c>
+      <x:c r="E28" s="28" t="str">
+        <x:v>Guard trước team mutation</x:v>
+      </x:c>
+      <x:c r="F28" s="28" t="str">
+        <x:v>Pending phải accept invitation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="48" hidden="0" customHeight="1">
+      <x:c r="A29" s="28" t="str">
+        <x:v>direct / inherited</x:v>
+      </x:c>
+      <x:c r="B29" s="28" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="C29" s="28" t="str">
+        <x:v>Membership khai báo trực tiếp hoặc nhận qua hierarchy</x:v>
+      </x:c>
+      <x:c r="D29" s="28" t="str">
+        <x:v>PoC chỉ quản lý direct</x:v>
+      </x:c>
+      <x:c r="E29" s="28" t="str">
+        <x:v>Nested teams</x:v>
+      </x:c>
+      <x:c r="F29" s="28" t="str">
+        <x:v>Remove direct có thể vẫn còn inherited</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="48" hidden="0" customHeight="1">
+      <x:c r="A30" s="28" t="str">
+        <x:v>ID / slug</x:v>
+      </x:c>
+      <x:c r="B30" s="28" t="str">
+        <x:v>GitHub</x:v>
+      </x:c>
+      <x:c r="C30" s="28" t="str">
+        <x:v>ID ổn định; slug thường theo name</x:v>
+      </x:c>
+      <x:c r="D30" s="28" t="str">
+        <x:v>ID giữ 19806617 khi rename</x:v>
+      </x:c>
+      <x:c r="E30" s="28" t="str">
+        <x:v>Reference và URL</x:v>
+      </x:c>
+      <x:c r="F30" s="28" t="str">
+        <x:v>Ưu tiên ID cho import</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31"/>
+    <x:row r="32"/>
+    <x:row r="33" ht="15" hidden="0" customHeight="1">
+      <x:c r="A33" s="23" t="str">
+        <x:v>Nguồn</x:v>
+      </x:c>
+      <x:c r="B33" s="23" t="str">
+        <x:v>URL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="36" hidden="0" customHeight="1">
+      <x:c r="A34" s="27" t="str">
+        <x:v>GitHub Provider</x:v>
+      </x:c>
+      <x:c r="B34" s="27" t="str">
+        <x:v>https://registry.terraform.io/providers/integrations/github/latest/docs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="48" hidden="0" customHeight="1">
+      <x:c r="A35" s="28" t="str">
+        <x:v>Organization membership resource</x:v>
+      </x:c>
+      <x:c r="B35" s="28" t="str">
+        <x:v>https://github.com/integrations/terraform-provider-github/blob/v6.13.0/docs/resources/membership.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="60" hidden="0" customHeight="1">
+      <x:c r="A36" s="28" t="str">
+        <x:v>Team membership resource</x:v>
+      </x:c>
+      <x:c r="B36" s="28" t="str">
+        <x:v>https://github.com/integrations/terraform-provider-github/blob/v6.13.0/docs/resources/team_membership.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="24" hidden="0" customHeight="1">
+      <x:c r="A37" s="28" t="str">
+        <x:v>GitHub organization/team API</x:v>
+      </x:c>
+      <x:c r="B37" s="28" t="str">
+        <x:v>https://docs.github.com/en/rest/orgs/members</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb8fcece26b474104"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>